<commit_message>
Allow cogs rate ranges in both forecast periods
</commit_message>
<xml_diff>
--- a/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル_一部目標未達.xlsx
+++ b/補助金/大規模成長投資補助金/planning_model/examples/成長投資計画_提案計画サンプル_一部目標未達.xlsx
@@ -204,7 +204,7 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <v>15.463873591495837</v>
+        <v>15.463655389422492</v>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
@@ -234,7 +234,7 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <v>9332089.869999997</v>
+        <v>9331938.869999997</v>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
@@ -264,7 +264,7 @@
         </is>
       </c>
       <c r="B10" s="2">
-        <v>2.184711746547996</v>
+        <v>2.1848118329287347</v>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
@@ -294,7 +294,7 @@
         </is>
       </c>
       <c r="B11" s="2">
-        <v>63.91256738860758</v>
+        <v>63.91236279520185</v>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
@@ -324,7 +324,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <v>22.020887065724626</v>
+        <v>22.02052627021196</v>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
@@ -354,7 +354,7 @@
         </is>
       </c>
       <c r="B13" s="2">
-        <v>7653023</v>
+        <v>7652872</v>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
@@ -384,7 +384,7 @@
         </is>
       </c>
       <c r="B14" s="2">
-        <v>25.09060099268099</v>
+        <v>23.15053074954352</v>
       </c>
       <c r="C14" s="0" t="inlineStr">
         <is>
@@ -414,7 +414,7 @@
         </is>
       </c>
       <c r="B15" s="2">
-        <v>1964757</v>
+        <v>1964723</v>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
@@ -444,7 +444,7 @@
         </is>
       </c>
       <c r="B16" s="2">
-        <v>7.009252613618577</v>
+        <v>7.00782348691229</v>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B17" s="2">
-        <v>222489.57999999996</v>
+        <v>269565.13</v>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B19" s="2">
-        <v>256.4956919060052</v>
+        <v>256.49125326370756</v>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
@@ -594,7 +594,7 @@
         </is>
       </c>
       <c r="B21" s="2">
-        <v>5.380301885516814</v>
+        <v>5.376457502612597</v>
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="B22" s="2">
-        <v>7976</v>
+        <v>7970</v>
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
@@ -1268,13 +1268,13 @@
         <v>17302362</v>
       </c>
       <c r="H3" s="4">
-        <v>19946039</v>
+        <v>19946005</v>
       </c>
       <c r="I3" s="4">
-        <v>22996374.97</v>
+        <v>22996292.97</v>
       </c>
       <c r="J3" s="4">
-        <v>26634451.869999997</v>
+        <v>26634300.869999997</v>
       </c>
     </row>
     <row r="4">
@@ -1304,13 +1304,13 @@
         <v>4.878010489642537</v>
       </c>
       <c r="H4" s="2">
-        <v>15.279283834195589</v>
+        <v>15.279087329232844</v>
       </c>
       <c r="I4" s="2">
-        <v>15.292940969382428</v>
+        <v>15.29272638806618</v>
       </c>
       <c r="J4" s="2">
-        <v>15.820219076902609</v>
+        <v>15.81997544015461</v>
       </c>
     </row>
     <row r="5">
@@ -1338,13 +1338,13 @@
         <v>11765605</v>
       </c>
       <c r="H5" s="2">
-        <v>13434963</v>
+        <v>13434940</v>
       </c>
       <c r="I5" s="2">
-        <v>15407469</v>
+        <v>15407414</v>
       </c>
       <c r="J5" s="2">
-        <v>17743999</v>
+        <v>17743899</v>
       </c>
     </row>
     <row r="6">
@@ -1406,13 +1406,13 @@
         <v>5536757</v>
       </c>
       <c r="H7" s="4">
-        <v>6511076</v>
+        <v>6511065</v>
       </c>
       <c r="I7" s="4">
-        <v>7588905.969999999</v>
+        <v>7588878.969999999</v>
       </c>
       <c r="J7" s="4">
-        <v>8890452.869999997</v>
+        <v>8890401.869999997</v>
       </c>
     </row>
     <row r="8">
@@ -1440,13 +1440,13 @@
         <v>32.00000670428697</v>
       </c>
       <c r="H8" s="2">
-        <v>32.643453670174814</v>
+        <v>32.64345416538299</v>
       </c>
       <c r="I8" s="2">
-        <v>33.00044454789128</v>
+        <v>33.00044481038806</v>
       </c>
       <c r="J8" s="2">
-        <v>33.37952255745069</v>
+        <v>33.37952031627702</v>
       </c>
     </row>
     <row r="9">
@@ -1465,22 +1465,22 @@
         <v>3640000</v>
       </c>
       <c r="E9" s="2">
-        <v>3828099</v>
+        <v>3828100</v>
       </c>
       <c r="F9" s="2">
-        <v>4029317</v>
+        <v>4029320</v>
       </c>
       <c r="G9" s="2">
-        <v>4242329</v>
+        <v>4242334</v>
       </c>
       <c r="H9" s="2">
-        <v>4619081</v>
+        <v>4619075</v>
       </c>
       <c r="I9" s="2">
-        <v>5073716.66</v>
+        <v>5094739.08</v>
       </c>
       <c r="J9" s="2">
-        <v>5583321.58</v>
+        <v>5630379.13</v>
       </c>
     </row>
     <row r="10">
@@ -1508,13 +1508,13 @@
         <v>114341</v>
       </c>
       <c r="H10" s="2">
-        <v>119899</v>
+        <v>119897</v>
       </c>
       <c r="I10" s="2">
-        <v>125729</v>
+        <v>125725</v>
       </c>
       <c r="J10" s="2">
-        <v>131844</v>
+        <v>131838</v>
       </c>
     </row>
     <row r="11">
@@ -1542,13 +1542,13 @@
         <v>102907</v>
       </c>
       <c r="H11" s="2">
-        <v>107909</v>
+        <v>107907</v>
       </c>
       <c r="I11" s="2">
-        <v>113156</v>
+        <v>113153</v>
       </c>
       <c r="J11" s="2">
-        <v>118660</v>
+        <v>118654</v>
       </c>
     </row>
     <row r="12">
@@ -1579,7 +1579,7 @@
         <v>11990</v>
       </c>
       <c r="I12" s="2">
-        <v>12573</v>
+        <v>12572</v>
       </c>
       <c r="J12" s="2">
         <v>13184</v>
@@ -1601,22 +1601,22 @@
         <v>1400000</v>
       </c>
       <c r="E13" s="2">
-        <v>1494027</v>
+        <v>1494028</v>
       </c>
       <c r="F13" s="2">
-        <v>1594417</v>
+        <v>1594420</v>
       </c>
       <c r="G13" s="2">
-        <v>1701607</v>
+        <v>1701612</v>
       </c>
       <c r="H13" s="2">
         <v>1817073</v>
       </c>
       <c r="I13" s="2">
-        <v>1974344.6600000001</v>
+        <v>1995380.08</v>
       </c>
       <c r="J13" s="2">
-        <v>2145739.58</v>
+        <v>2192820.13</v>
       </c>
     </row>
     <row r="14">
@@ -1635,22 +1635,22 @@
         <v>1330000</v>
       </c>
       <c r="E14" s="2">
-        <v>1419325</v>
+        <v>1419326</v>
       </c>
       <c r="F14" s="2">
-        <v>1514696</v>
+        <v>1514699</v>
       </c>
       <c r="G14" s="2">
-        <v>1616526</v>
+        <v>1616531</v>
       </c>
       <c r="H14" s="2">
-        <v>1756553</v>
+        <v>1775364</v>
       </c>
       <c r="I14" s="2">
-        <v>1909168</v>
+        <v>1951260</v>
       </c>
       <c r="J14" s="2">
-        <v>2075539</v>
+        <v>2146192</v>
       </c>
     </row>
     <row r="15">
@@ -1678,13 +1678,13 @@
         <v>85081</v>
       </c>
       <c r="H15" s="2">
-        <v>92451</v>
+        <v>93441</v>
       </c>
       <c r="I15" s="2">
-        <v>100483</v>
+        <v>102698</v>
       </c>
       <c r="J15" s="2">
-        <v>109239</v>
+        <v>112958</v>
       </c>
     </row>
     <row r="16">
@@ -1752,7 +1752,7 @@
         <v>105579</v>
       </c>
       <c r="J17" s="2">
-        <v>123181</v>
+        <v>123180</v>
       </c>
     </row>
     <row r="18">
@@ -1771,22 +1771,22 @@
         <v>1160000</v>
       </c>
       <c r="E18" s="4">
-        <v>1205743</v>
+        <v>1205742</v>
       </c>
       <c r="F18" s="4">
-        <v>1249917</v>
+        <v>1249914</v>
       </c>
       <c r="G18" s="4">
-        <v>1294428</v>
+        <v>1294423</v>
       </c>
       <c r="H18" s="4">
-        <v>1891995</v>
+        <v>1891990</v>
       </c>
       <c r="I18" s="4">
-        <v>2515189.3099999987</v>
+        <v>2494139.8899999987</v>
       </c>
       <c r="J18" s="4">
-        <v>3307131.2899999972</v>
+        <v>3260022.7399999974</v>
       </c>
     </row>
     <row r="19">
@@ -1805,22 +1805,22 @@
         <v>7.733333333333333</v>
       </c>
       <c r="E19" s="2">
-        <v>7.664876373392353</v>
+        <v>7.664870016418791</v>
       </c>
       <c r="F19" s="2">
-        <v>7.576353346276221</v>
+        <v>7.576335161820742</v>
       </c>
       <c r="G19" s="2">
-        <v>7.481221350009901</v>
+        <v>7.481192452221263</v>
       </c>
       <c r="H19" s="2">
-        <v>9.485567535489126</v>
+        <v>9.485558636930051</v>
       </c>
       <c r="I19" s="2">
-        <v>10.937329528159102</v>
+        <v>10.84583455800354</v>
       </c>
       <c r="J19" s="2">
-        <v>12.416742443740771</v>
+        <v>12.23994110418712</v>
       </c>
     </row>
     <row r="20">
@@ -1839,22 +1839,22 @@
         <v>1130000</v>
       </c>
       <c r="E20" s="4">
-        <v>1169253</v>
+        <v>1169252</v>
       </c>
       <c r="F20" s="4">
-        <v>1211873</v>
+        <v>1211870</v>
       </c>
       <c r="G20" s="4">
-        <v>1254765</v>
+        <v>1254760</v>
       </c>
       <c r="H20" s="4">
-        <v>1733905</v>
+        <v>1714099</v>
       </c>
       <c r="I20" s="4">
-        <v>2345830</v>
+        <v>2301509</v>
       </c>
       <c r="J20" s="4">
-        <v>3125652</v>
+        <v>3051252</v>
       </c>
     </row>
     <row r="21">
@@ -1873,22 +1873,22 @@
         <v>1130000</v>
       </c>
       <c r="E21" s="2">
-        <v>1169253</v>
+        <v>1169252</v>
       </c>
       <c r="F21" s="2">
-        <v>1211873</v>
+        <v>1211870</v>
       </c>
       <c r="G21" s="2">
-        <v>1254765</v>
+        <v>1254760</v>
       </c>
       <c r="H21" s="2">
-        <v>1733905</v>
+        <v>1714099</v>
       </c>
       <c r="I21" s="2">
-        <v>2345830</v>
+        <v>2301509</v>
       </c>
       <c r="J21" s="2">
-        <v>3125652</v>
+        <v>3051252</v>
       </c>
     </row>
     <row r="22">
@@ -1910,19 +1910,19 @@
         <v>818477</v>
       </c>
       <c r="F22" s="2">
-        <v>848312</v>
+        <v>848310</v>
       </c>
       <c r="G22" s="2">
-        <v>878336</v>
+        <v>878332</v>
       </c>
       <c r="H22" s="2">
-        <v>1213734</v>
+        <v>1199869</v>
       </c>
       <c r="I22" s="2">
-        <v>1642081</v>
+        <v>1611057</v>
       </c>
       <c r="J22" s="2">
-        <v>2187957</v>
+        <v>2135877</v>
       </c>
     </row>
     <row r="23">
@@ -1941,22 +1941,22 @@
         <v>1400000</v>
       </c>
       <c r="E23" s="2">
-        <v>1494027</v>
+        <v>1494028</v>
       </c>
       <c r="F23" s="2">
-        <v>1594417</v>
+        <v>1594420</v>
       </c>
       <c r="G23" s="2">
-        <v>1701607</v>
+        <v>1701612</v>
       </c>
       <c r="H23" s="2">
         <v>1817073</v>
       </c>
       <c r="I23" s="2">
-        <v>1974344.6600000001</v>
+        <v>1995380.08</v>
       </c>
       <c r="J23" s="2">
-        <v>2145739.58</v>
+        <v>2192820.13</v>
       </c>
     </row>
     <row r="24">
@@ -1984,13 +1984,13 @@
         <v>114341</v>
       </c>
       <c r="H24" s="2">
-        <v>119899</v>
+        <v>119897</v>
       </c>
       <c r="I24" s="2">
-        <v>125729</v>
+        <v>125725</v>
       </c>
       <c r="J24" s="2">
-        <v>131844</v>
+        <v>131838</v>
       </c>
     </row>
     <row r="25">
@@ -2052,13 +2052,13 @@
         <v>3460376</v>
       </c>
       <c r="H26" s="4">
-        <v>4178967</v>
+        <v>4178960</v>
       </c>
       <c r="I26" s="4">
-        <v>4965262.969999999</v>
+        <v>4965244.969999999</v>
       </c>
       <c r="J26" s="4">
-        <v>5934714.869999997</v>
+        <v>5934680.869999997</v>
       </c>
     </row>
     <row r="27">
@@ -2088,13 +2088,13 @@
         <v>4.743232914859963</v>
       </c>
       <c r="H27" s="2">
-        <v>20.766269330269303</v>
+        <v>20.76606704011357</v>
       </c>
       <c r="I27" s="2">
-        <v>18.81555824681074</v>
+        <v>18.815326540574652</v>
       </c>
       <c r="J27" s="2">
-        <v>19.524683906117435</v>
+        <v>19.52443244708626</v>
       </c>
     </row>
     <row r="28">
@@ -2122,13 +2122,13 @@
         <v>19.999442850635074</v>
       </c>
       <c r="H28" s="2">
-        <v>20.951362824468557</v>
+        <v>20.951363443456472</v>
       </c>
       <c r="I28" s="2">
-        <v>21.59150290633828</v>
+        <v>21.591501623663646</v>
       </c>
       <c r="J28" s="2">
-        <v>22.282098760532882</v>
+        <v>22.282097431303807</v>
       </c>
     </row>
     <row r="29">
@@ -2156,13 +2156,13 @@
         <v>262</v>
       </c>
       <c r="H29" s="2">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="I29" s="2">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="J29" s="2">
-        <v>291</v>
+        <v>297</v>
       </c>
     </row>
     <row r="30">
@@ -2215,22 +2215,22 @@
         <v>6086.95652173913</v>
       </c>
       <c r="E31" s="2">
-        <v>6225.1125</v>
+        <v>6225.116666666667</v>
       </c>
       <c r="F31" s="2">
-        <v>6327.0515873015875</v>
+        <v>6327.063492063492</v>
       </c>
       <c r="G31" s="2">
-        <v>6494.68320610687</v>
+        <v>6494.702290076336</v>
       </c>
       <c r="H31" s="2">
-        <v>6705.066420664207</v>
+        <v>6655.945054945055</v>
       </c>
       <c r="I31" s="2">
-        <v>7026.137580071175</v>
+        <v>7001.333614035088</v>
       </c>
       <c r="J31" s="2">
-        <v>7373.675532646048</v>
+        <v>7383.23276094276</v>
       </c>
     </row>
     <row r="32">
@@ -2251,22 +2251,22 @@
         <v>1.9923071308914908</v>
       </c>
       <c r="E32" s="2">
-        <v>2.2697053571428594</v>
+        <v>2.269773809523823</v>
       </c>
       <c r="F32" s="2">
-        <v>1.6375461054171758</v>
+        <v>1.6376693137771126</v>
       </c>
       <c r="G32" s="2">
-        <v>2.6494428959883853</v>
+        <v>2.6495513791370273</v>
       </c>
       <c r="H32" s="2">
-        <v>3.2393144958866804</v>
+        <v>2.48268138656782</v>
       </c>
       <c r="I32" s="2">
-        <v>4.788485889080318</v>
+        <v>5.1891738323985415</v>
       </c>
       <c r="J32" s="2">
-        <v>4.946358488063551</v>
+        <v>5.45466289653882</v>
       </c>
     </row>
     <row r="33">
@@ -2294,13 +2294,13 @@
         <v>22868.2</v>
       </c>
       <c r="H33" s="2">
-        <v>23979.8</v>
+        <v>23979.4</v>
       </c>
       <c r="I33" s="2">
-        <v>25145.8</v>
+        <v>25145</v>
       </c>
       <c r="J33" s="2">
-        <v>26368.8</v>
+        <v>26367.6</v>
       </c>
     </row>
     <row r="34">
@@ -2330,13 +2330,13 @@
         <v>4.572850074537449</v>
       </c>
       <c r="H34" s="2">
-        <v>4.860898540331116</v>
+        <v>4.859149386484285</v>
       </c>
       <c r="I34" s="2">
-        <v>4.862425875111542</v>
+        <v>4.860838886711094</v>
       </c>
       <c r="J34" s="2">
-        <v>4.863635279052558</v>
+        <v>4.862199244382581</v>
       </c>
     </row>
     <row r="35">
@@ -2364,13 +2364,13 @@
         <v>12960.209737827716</v>
       </c>
       <c r="H35" s="2">
-        <v>15141.184782608696</v>
+        <v>15032.230215827338</v>
       </c>
       <c r="I35" s="2">
-        <v>17361.059335664333</v>
+        <v>17121.534379310342</v>
       </c>
       <c r="J35" s="2">
-        <v>20049.71239864864</v>
+        <v>19651.26115894039</v>
       </c>
     </row>
     <row r="36">
@@ -2389,22 +2389,22 @@
         <v>1510000</v>
       </c>
       <c r="E36" s="4">
-        <v>1555743</v>
+        <v>1555742</v>
       </c>
       <c r="F36" s="4">
-        <v>1599917</v>
+        <v>1599914</v>
       </c>
       <c r="G36" s="4">
-        <v>1644428</v>
+        <v>1644423</v>
       </c>
       <c r="H36" s="4">
-        <v>2241995</v>
+        <v>2241990</v>
       </c>
       <c r="I36" s="4">
-        <v>2865189.3099999987</v>
+        <v>2844139.8899999987</v>
       </c>
       <c r="J36" s="4">
-        <v>3657131.2899999972</v>
+        <v>3610022.7399999974</v>
       </c>
     </row>
     <row r="37">
@@ -2423,22 +2423,22 @@
         <v>10.066666666666666</v>
       </c>
       <c r="E37" s="2">
-        <v>9.889817120041783</v>
+        <v>9.88981076306822</v>
       </c>
       <c r="F37" s="2">
-        <v>9.697873152148674</v>
+        <v>9.697854967693194</v>
       </c>
       <c r="G37" s="2">
-        <v>9.504066554612601</v>
+        <v>9.504037656823964</v>
       </c>
       <c r="H37" s="2">
-        <v>11.240301896531937</v>
+        <v>11.240295989096563</v>
       </c>
       <c r="I37" s="2">
-        <v>12.45930853770558</v>
+        <v>12.36781899461076</v>
       </c>
       <c r="J37" s="2">
-        <v>13.730829933538999</v>
+        <v>13.55403604404803</v>
       </c>
     </row>
     <row r="38">
@@ -2459,22 +2459,22 @@
         <v>3.0486007228415657</v>
       </c>
       <c r="E38" s="2">
-        <v>3.029337748344374</v>
+        <v>3.0292715231788003</v>
       </c>
       <c r="F38" s="2">
-        <v>2.839414993350453</v>
+        <v>2.8392882624496796</v>
       </c>
       <c r="G38" s="2">
-        <v>2.782081820494442</v>
+        <v>2.7819620304591286</v>
       </c>
       <c r="H38" s="2">
-        <v>36.338897172755516</v>
+        <v>36.339007664086424</v>
       </c>
       <c r="I38" s="2">
-        <v>27.79641836846196</v>
+        <v>26.8578312124496</v>
       </c>
       <c r="J38" s="2">
-        <v>27.640127555829764</v>
+        <v>26.928452172582794</v>
       </c>
     </row>
   </sheetData>
@@ -2636,13 +2636,13 @@
         <v>9369739</v>
       </c>
       <c r="H3" s="4">
-        <v>11433039</v>
+        <v>11433005</v>
       </c>
       <c r="I3" s="4">
-        <v>13950695</v>
+        <v>13950613</v>
       </c>
       <c r="J3" s="4">
-        <v>17022762</v>
+        <v>17022611</v>
       </c>
     </row>
     <row r="4">
@@ -2672,13 +2672,13 @@
         <v>5.409360836980381</v>
       </c>
       <c r="H4" s="2">
-        <v>22.02089087006587</v>
+        <v>22.02052799976606</v>
       </c>
       <c r="I4" s="2">
-        <v>22.02088176205819</v>
+        <v>22.02052741164724</v>
       </c>
       <c r="J4" s="2">
-        <v>22.02088856504998</v>
+        <v>22.020523399222668</v>
       </c>
     </row>
     <row r="5">
@@ -2706,13 +2706,13 @@
         <v>54.15294744151117</v>
       </c>
       <c r="H5" s="2">
-        <v>57.31984681269299</v>
+        <v>57.31977406001854</v>
       </c>
       <c r="I5" s="2">
-        <v>60.66475702452855</v>
+        <v>60.66461676322956</v>
       </c>
       <c r="J5" s="2">
-        <v>63.91256738860758</v>
+        <v>63.91236279520185</v>
       </c>
     </row>
     <row r="6">
@@ -2740,13 +2740,13 @@
         <v>2998317</v>
       </c>
       <c r="H6" s="4">
-        <v>3715738</v>
+        <v>3715727</v>
       </c>
       <c r="I6" s="4">
-        <v>4603729</v>
+        <v>4603702</v>
       </c>
       <c r="J6" s="4">
-        <v>5702625</v>
+        <v>5702574</v>
       </c>
     </row>
     <row r="7">
@@ -2774,13 +2774,13 @@
         <v>32.00000554978106</v>
       </c>
       <c r="H7" s="2">
-        <v>32.50000284263878</v>
+        <v>32.50000327997758</v>
       </c>
       <c r="I7" s="2">
-        <v>32.999997491164414</v>
+        <v>32.9999979212383</v>
       </c>
       <c r="J7" s="2">
-        <v>33.49999841388841</v>
+        <v>33.49999597594047</v>
       </c>
     </row>
     <row r="8">
@@ -2799,22 +2799,22 @@
         <v>730000</v>
       </c>
       <c r="E8" s="4">
-        <v>765642</v>
+        <v>765641</v>
       </c>
       <c r="F8" s="4">
-        <v>802328</v>
+        <v>802325</v>
       </c>
       <c r="G8" s="4">
-        <v>840048</v>
+        <v>840043</v>
       </c>
       <c r="H8" s="4">
-        <v>1297239</v>
+        <v>1297234</v>
       </c>
       <c r="I8" s="4">
-        <v>1854112.3399999999</v>
+        <v>1833062.92</v>
       </c>
       <c r="J8" s="4">
-        <v>2574339.42</v>
+        <v>2527230.87</v>
       </c>
     </row>
     <row r="9">
@@ -2833,22 +2833,22 @@
         <v>9.125</v>
       </c>
       <c r="E9" s="2">
-        <v>9.07938799079636</v>
+        <v>9.079376132267189</v>
       </c>
       <c r="F9" s="2">
-        <v>9.026172624617699</v>
+        <v>9.026138874682667</v>
       </c>
       <c r="G9" s="2">
-        <v>8.96554322377603</v>
+        <v>8.965489860496648</v>
       </c>
       <c r="H9" s="2">
-        <v>11.346405798143433</v>
+        <v>11.346395807576398</v>
       </c>
       <c r="I9" s="2">
-        <v>13.290465743821365</v>
+        <v>13.139658594213744</v>
       </c>
       <c r="J9" s="2">
-        <v>15.12292435269905</v>
+        <v>14.846317465634385</v>
       </c>
     </row>
     <row r="10">
@@ -2867,22 +2867,22 @@
         <v>600000</v>
       </c>
       <c r="E10" s="2">
-        <v>644416</v>
+        <v>644417</v>
       </c>
       <c r="F10" s="2">
-        <v>692119</v>
+        <v>692122</v>
       </c>
       <c r="G10" s="2">
-        <v>743354</v>
+        <v>743359</v>
       </c>
       <c r="H10" s="2">
         <v>790000</v>
       </c>
       <c r="I10" s="2">
-        <v>873508.66</v>
+        <v>894544.08</v>
       </c>
       <c r="J10" s="2">
-        <v>965843.58</v>
+        <v>1012924.13</v>
       </c>
     </row>
     <row r="11">
@@ -2910,13 +2910,13 @@
         <v>46849</v>
       </c>
       <c r="H11" s="2">
-        <v>49370</v>
+        <v>49368</v>
       </c>
       <c r="I11" s="2">
-        <v>52026</v>
+        <v>52022</v>
       </c>
       <c r="J11" s="2">
-        <v>54825</v>
+        <v>54819</v>
       </c>
     </row>
     <row r="12">
@@ -3046,13 +3046,13 @@
         <v>1830251</v>
       </c>
       <c r="H15" s="4">
-        <v>2336609</v>
+        <v>2336602</v>
       </c>
       <c r="I15" s="4">
-        <v>2979647</v>
+        <v>2979629</v>
       </c>
       <c r="J15" s="4">
-        <v>3795008</v>
+        <v>3794974</v>
       </c>
     </row>
     <row r="16">
@@ -3082,13 +3082,13 @@
         <v>5.253862804590503</v>
       </c>
       <c r="H16" s="2">
-        <v>27.66604143366129</v>
+        <v>27.665658972457873</v>
       </c>
       <c r="I16" s="2">
-        <v>27.520137087548658</v>
+        <v>27.519748763375198</v>
       </c>
       <c r="J16" s="2">
-        <v>27.364348864143984</v>
+        <v>27.36397719313377</v>
       </c>
     </row>
     <row r="17">
@@ -3116,13 +3116,13 @@
         <v>116</v>
       </c>
       <c r="H17" s="2">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="I17" s="2">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="J17" s="2">
-        <v>123</v>
+        <v>129</v>
       </c>
     </row>
     <row r="18">
@@ -3175,22 +3175,22 @@
         <v>6000</v>
       </c>
       <c r="E19" s="2">
-        <v>6137.295238095238</v>
+        <v>6137.304761904762</v>
       </c>
       <c r="F19" s="2">
-        <v>6235.306306306306</v>
+        <v>6235.333333333333</v>
       </c>
       <c r="G19" s="2">
-        <v>6408.224137931034</v>
+        <v>6408.267241379311</v>
       </c>
       <c r="H19" s="2">
-        <v>6694.9152542372885</v>
+        <v>6583.333333333333</v>
       </c>
       <c r="I19" s="2">
-        <v>7219.079834710744</v>
+        <v>7156.35264</v>
       </c>
       <c r="J19" s="2">
-        <v>7852.386829268293</v>
+        <v>7852.12503875969</v>
       </c>
     </row>
     <row r="20">
@@ -3211,22 +3211,22 @@
         <v>1.9999141053354874</v>
       </c>
       <c r="E20" s="2">
-        <v>2.2882539682539615</v>
+        <v>2.2884126984126896</v>
       </c>
       <c r="F20" s="2">
-        <v>1.5969749606096206</v>
+        <v>1.5972576763182866</v>
       </c>
       <c r="G20" s="2">
-        <v>2.7732050861694058</v>
+        <v>2.773450893499052</v>
       </c>
       <c r="H20" s="2">
-        <v>4.473799763171438</v>
+        <v>2.7318787647242493</v>
       </c>
       <c r="I20" s="2">
-        <v>7.829293733654152</v>
+        <v>8.704090734177218</v>
       </c>
       <c r="J20" s="2">
-        <v>8.772683071220321</v>
+        <v>9.722444291952748</v>
       </c>
     </row>
     <row r="21">
@@ -3254,13 +3254,13 @@
         <v>23424.5</v>
       </c>
       <c r="H21" s="2">
-        <v>24685</v>
+        <v>24684</v>
       </c>
       <c r="I21" s="2">
-        <v>26013</v>
+        <v>26011</v>
       </c>
       <c r="J21" s="2">
-        <v>27412.5</v>
+        <v>27409.5</v>
       </c>
     </row>
     <row r="22">
@@ -3290,13 +3290,13 @@
         <v>5.408932388345145</v>
       </c>
       <c r="H22" s="2">
-        <v>5.381118060150691</v>
+        <v>5.376849025592856</v>
       </c>
       <c r="I22" s="2">
-        <v>5.379785294713391</v>
+        <v>5.375952033706044</v>
       </c>
       <c r="J22" s="2">
-        <v>5.380002306539033</v>
+        <v>5.376571450540157</v>
       </c>
     </row>
     <row r="23">
@@ -3324,13 +3324,13 @@
         <v>15510.601694915254</v>
       </c>
       <c r="H23" s="2">
-        <v>19471.741666666665</v>
+        <v>19152.475409836065</v>
       </c>
       <c r="I23" s="2">
-        <v>24224.772357723577</v>
+        <v>23461.645669291338</v>
       </c>
       <c r="J23" s="2">
-        <v>30360.064</v>
+        <v>28969.26717557252</v>
       </c>
     </row>
     <row r="24">
@@ -3849,12 +3849,12 @@
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 22.06 % / 補助 19.71 % / ベース 25.69 %</t>
+          <t xml:space="preserve">全社 22.15 % / 補助 19.86 % / ベース 25.69 %</t>
         </is>
       </c>
       <c r="L7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 20.96 % / 補助 18.38 % / ベース 25.54 %</t>
+          <t xml:space="preserve">全社 21.14 % / 補助 18.65 % / ベース 25.54 %</t>
         </is>
       </c>
     </row>
@@ -3911,12 +3911,12 @@
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.94 % / 補助 13.29 % / ベース 7.31 %</t>
+          <t xml:space="preserve">全社 10.85 % / 補助 13.14 % / ベース 7.31 %</t>
         </is>
       </c>
       <c r="L8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.42 % / 補助 15.12 % / ベース 7.62 %</t>
+          <t xml:space="preserve">全社 12.24 % / 補助 14.85 % / ベース 7.62 %</t>
         </is>
       </c>
     </row>
@@ -3973,12 +3973,12 @@
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.46 % / 補助 14.72 % / ベース 8.97 %</t>
+          <t xml:space="preserve">全社 12.37 % / 補助 14.57 % / ベース 8.97 %</t>
         </is>
       </c>
       <c r="L9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 13.73 % / 補助 16.3 % / ベース 9.18 %</t>
+          <t xml:space="preserve">全社 13.55 % / 補助 16.02 % / ベース 9.18 %</t>
         </is>
       </c>
     </row>
@@ -4159,12 +4159,12 @@
       </c>
       <c r="K12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.59 % / 補助 6.26 % / ベース 12.17 %</t>
+          <t xml:space="preserve">全社 8.68 % / 補助 6.41 % / ベース 12.17 %</t>
         </is>
       </c>
       <c r="L12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.06 % / 補助 5.67 % / ベース 12.28 %</t>
+          <t xml:space="preserve">全社 8.23 % / 補助 5.95 % / ベース 12.28 %</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
       </c>
       <c r="L13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 0.5 % / 補助 0.32 % / ベース 0.8 %</t>
+          <t xml:space="preserve">全社 0.49 % / 補助 0.32 % / ベース 0.8 %</t>
         </is>
       </c>
     </row>
@@ -4283,12 +4283,12 @@
       </c>
       <c r="K14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 9.13 % / 補助 6.63 % / ベース 12.98 %</t>
+          <t xml:space="preserve">全社 9.22 % / 補助 6.79 % / ベース 12.98 %</t>
         </is>
       </c>
       <c r="L14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.55 % / 補助 6 % / ベース 13.08 %</t>
+          <t xml:space="preserve">全社 8.73 % / 補助 6.27 % / ベース 13.08 %</t>
         </is>
       </c>
     </row>
@@ -4325,32 +4325,32 @@
       </c>
       <c r="G15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6,225.11 千円/人 / 補助 6,137.3 千円/人 / ベース 6,293.41 千円/人</t>
+          <t xml:space="preserve">全社 6,225.12 千円/人 / 補助 6,137.3 千円/人 / ベース 6,293.41 千円/人</t>
         </is>
       </c>
       <c r="H15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6,327.05 千円/人 / 補助 6,235.31 千円/人 / ベース 6,399.28 千円/人</t>
+          <t xml:space="preserve">全社 6,327.06 千円/人 / 補助 6,235.33 千円/人 / ベース 6,399.28 千円/人</t>
         </is>
       </c>
       <c r="I15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6,494.68 千円/人 / 補助 6,408.22 千円/人 / ベース 6,563.38 千円/人</t>
+          <t xml:space="preserve">全社 6,494.7 千円/人 / 補助 6,408.27 千円/人 / ベース 6,563.38 千円/人</t>
         </is>
       </c>
       <c r="J15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6,705.07 千円/人 / 補助 6,694.92 千円/人 / ベース 6,712.9 千円/人</t>
+          <t xml:space="preserve">全社 6,655.95 千円/人 / 補助 6,583.33 千円/人 / ベース 6,712.9 千円/人</t>
         </is>
       </c>
       <c r="K15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7,026.14 千円/人 / 補助 7,219.08 千円/人 / ベース 6,880.23 千円/人</t>
+          <t xml:space="preserve">全社 7,001.33 千円/人 / 補助 7,156.35 千円/人 / ベース 6,880.23 千円/人</t>
         </is>
       </c>
       <c r="L15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 7,373.68 千円/人 / 補助 7,852.39 千円/人 / ベース 7,023.19 千円/人</t>
+          <t xml:space="preserve">全社 7,383.23 千円/人 / 補助 7,852.13 千円/人 / ベース 7,023.19 千円/人</t>
         </is>
       </c>
     </row>
@@ -4402,17 +4402,17 @@
       </c>
       <c r="J16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 23,979.8 千円/人 / 補助 24,685 千円/人 / ベース 23,509.67 千円/人</t>
+          <t xml:space="preserve">全社 23,979.4 千円/人 / 補助 24,684 千円/人 / ベース 23,509.67 千円/人</t>
         </is>
       </c>
       <c r="K16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 25,145.8 千円/人 / 補助 26,013 千円/人 / ベース 24,567.67 千円/人</t>
+          <t xml:space="preserve">全社 25,145 千円/人 / 補助 26,011 千円/人 / ベース 24,567.67 千円/人</t>
         </is>
       </c>
       <c r="L16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 26,368.8 千円/人 / 補助 27,412.5 千円/人 / ベース 25,673 千円/人</t>
+          <t xml:space="preserve">全社 26,367.6 千円/人 / 補助 27,409.5 千円/人 / ベース 25,673 千円/人</t>
         </is>
       </c>
     </row>
@@ -4464,17 +4464,17 @@
       </c>
       <c r="J17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.24 % / 補助 4.47 % / ベース 2.28 %</t>
+          <t xml:space="preserve">全社 2.48 % / 補助 2.73 % / ベース 2.28 %</t>
         </is>
       </c>
       <c r="K17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.79 % / 補助 7.83 % / ベース 2.49 %</t>
+          <t xml:space="preserve">全社 5.19 % / 補助 8.7 % / ベース 2.49 %</t>
         </is>
       </c>
       <c r="L17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4.95 % / 補助 8.77 % / ベース 2.08 %</t>
+          <t xml:space="preserve">全社 5.45 % / 補助 9.72 % / ベース 2.08 %</t>
         </is>
       </c>
     </row>
@@ -4511,7 +4511,7 @@
       </c>
       <c r="G18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 50.68 % / 補助 41.55 % / ベース 60.72 %</t>
+          <t xml:space="preserve">全社 50.68 % / 補助 41.56 % / ベース 60.72 %</t>
         </is>
       </c>
       <c r="H18" s="0" t="inlineStr">
@@ -4531,12 +4531,12 @@
       </c>
       <c r="K18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 42.3 % / 補助 31.06 % / ベース 59.15 %</t>
+          <t xml:space="preserve">全社 42.72 % / 補助 31.77 % / ベース 59.15 %</t>
         </is>
       </c>
       <c r="L18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 38.38 % / 補助 26.9 % / ベース 58.74 %</t>
+          <t xml:space="preserve">全社 39.17 % / 補助 28.14 % / ベース 58.74 %</t>
         </is>
       </c>
     </row>
@@ -4650,17 +4650,17 @@
       </c>
       <c r="J20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 73,601.62 千円/人 / 補助 96,890.16 千円/人 / ベース 55,640.52 千円/人</t>
+          <t xml:space="preserve">全社 73,062.29 千円/人 / 補助 95,275.04 千円/人 / ベース 55,640.52 千円/人</t>
         </is>
       </c>
       <c r="K20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 81,837.63 千円/人 / 補助 115,295 千円/人 / ベース 56,535.5 千円/人</t>
+          <t xml:space="preserve">全社 80,688.75 千円/人 / 補助 111,604.9 千円/人 / ベース 56,535.5 千円/人</t>
         </is>
       </c>
       <c r="L20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 91,527.33 千円/人 / 補助 138,396.44 千円/人 / ベース 57,212.44 千円/人</t>
+          <t xml:space="preserve">全社 89,677.78 千円/人 / 補助 131,958.22 千円/人 / ベース 57,212.44 千円/人</t>
         </is>
       </c>
     </row>
@@ -4697,32 +4697,32 @@
       </c>
       <c r="G21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 5,023.93 千円/人 / 補助 7,291.83 千円/人 / ベース 3,260.01 千円/人</t>
+          <t xml:space="preserve">全社 5,023.93 千円/人 / 補助 7,291.82 千円/人 / ベース 3,260.01 千円/人</t>
         </is>
       </c>
       <c r="H21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4,959.99 千円/人 / 補助 7,228.18 千円/人 / ベース 3,174.39 千円/人</t>
+          <t xml:space="preserve">全社 4,959.98 千円/人 / 補助 7,228.15 千円/人 / ベース 3,174.39 千円/人</t>
         </is>
       </c>
       <c r="I21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 4,940.56 千円/人 / 補助 7,241.79 千円/人 / ベース 3,112.19 千円/人</t>
+          <t xml:space="preserve">全社 4,940.55 千円/人 / 補助 7,241.75 千円/人 / ベース 3,112.19 千円/人</t>
         </is>
       </c>
       <c r="J21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 6,981.53 千円/人 / 補助 10,993.55 千円/人 / ベース 3,887.29 千円/人</t>
+          <t xml:space="preserve">全社 6,930.37 千円/人 / 補助 10,810.28 千円/人 / ベース 3,887.29 千円/人</t>
         </is>
       </c>
       <c r="K21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8,950.85 千円/人 / 補助 15,323.24 千円/人 / ベース 4,131.73 千円/人</t>
+          <t xml:space="preserve">全社 8,751.37 千円/人 / 補助 14,664.5 千円/人 / ベース 4,131.73 千円/人</t>
         </is>
       </c>
       <c r="L21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11,364.71 千円/人 / 補助 20,929.59 千円/人 / ベース 4,361.86 千円/人</t>
+          <t xml:space="preserve">全社 10,976.51 千円/人 / 補助 19,590.94 千円/人 / ベース 4,361.86 千円/人</t>
         </is>
       </c>
     </row>
@@ -4774,17 +4774,17 @@
       </c>
       <c r="J22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 15,141.18 千円/人 / 補助 19,471.74 千円/人 / ベース 11,809.99 千円/人</t>
+          <t xml:space="preserve">全社 15,032.23 千円/人 / 補助 19,152.48 千円/人 / ベース 11,809.99 千円/人</t>
         </is>
       </c>
       <c r="K22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 17,361.06 千円/人 / 補助 24,224.77 千円/人 / ベース 12,181.69 千円/人</t>
+          <t xml:space="preserve">全社 17,121.53 千円/人 / 補助 23,461.65 千円/人 / ベース 12,181.69 千円/人</t>
         </is>
       </c>
       <c r="L22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 20,049.71 千円/人 / 補助 30,360.06 千円/人 / ベース 12,512.91 千円/人</t>
+          <t xml:space="preserve">全社 19,651.26 千円/人 / 補助 28,969.27 千円/人 / ベース 12,512.91 千円/人</t>
         </is>
       </c>
     </row>
@@ -4836,17 +4836,17 @@
       </c>
       <c r="J23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.44 % / 補助 1.72 % / ベース 4.79 %</t>
+          <t xml:space="preserve">全社 4.2 % / 補助 3.45 % / ベース 4.79 %</t>
         </is>
       </c>
       <c r="K23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.69 % / 補助 2.54 % / ベース 4.58 %</t>
+          <t xml:space="preserve">全社 4.4 % / 補助 4.17 % / ベース 4.58 %</t>
         </is>
       </c>
       <c r="L23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 3.56 % / 補助 1.65 % / ベース 5 %</t>
+          <t xml:space="preserve">全社 4.21 % / 補助 3.2 % / ベース 5 %</t>
         </is>
       </c>
     </row>
@@ -4898,17 +4898,17 @@
       </c>
       <c r="J24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.84 pt / 補助 20.3 pt / ベース 2.52 pt</t>
+          <t xml:space="preserve">全社 11.08 pt / 補助 18.57 pt / ベース 2.52 pt</t>
         </is>
       </c>
       <c r="K24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 11.6 pt / 補助 19.48 pt / ベース 1.68 pt</t>
+          <t xml:space="preserve">全社 10.9 pt / 補助 17.85 pt / ベース 1.68 pt</t>
         </is>
       </c>
       <c r="L24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 12.26 pt / 補助 20.37 pt / ベース 1.26 pt</t>
+          <t xml:space="preserve">全社 11.61 pt / 補助 18.82 pt / ベース 1.26 pt</t>
         </is>
       </c>
     </row>
@@ -5213,12 +5213,12 @@
       </c>
       <c r="K29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 8.19 倍 / 補助 10.27 倍 / ベース 5.41 倍</t>
+          <t xml:space="preserve">全社 8.13 倍 / 補助 10.17 倍 / ベース 5.41 倍</t>
         </is>
       </c>
       <c r="L29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">全社 10.45 倍 / 補助 13.87 倍 / ベース 5.89 倍</t>
+          <t xml:space="preserve">全社 10.31 倍 / 補助 13.64 倍 / ベース 5.89 倍</t>
         </is>
       </c>
     </row>
@@ -5585,12 +5585,12 @@
       </c>
       <c r="K35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 5.98 pt</t>
+          <t xml:space="preserve">差 5.83 pt</t>
         </is>
       </c>
       <c r="L35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">差 7.5 pt</t>
+          <t xml:space="preserve">差 7.22 pt</t>
         </is>
       </c>
     </row>
@@ -5642,17 +5642,17 @@
       </c>
       <c r="J36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 96,890.16 千円/人 / ベース 55,640.52 千円/人</t>
+          <t xml:space="preserve">補助 95,275.04 千円/人 / ベース 55,640.52 千円/人</t>
         </is>
       </c>
       <c r="K36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 115,295 千円/人 / ベース 56,535.5 千円/人</t>
+          <t xml:space="preserve">補助 111,604.9 千円/人 / ベース 56,535.5 千円/人</t>
         </is>
       </c>
       <c r="L36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 138,396.44 千円/人 / ベース 57,212.44 千円/人</t>
+          <t xml:space="preserve">補助 131,958.22 千円/人 / ベース 57,212.44 千円/人</t>
         </is>
       </c>
     </row>
@@ -5694,27 +5694,27 @@
       </c>
       <c r="H37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 6,235.31 千円/人 / ベース 6,399.28 千円/人</t>
+          <t xml:space="preserve">補助 6,235.33 千円/人 / ベース 6,399.28 千円/人</t>
         </is>
       </c>
       <c r="I37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 6,408.22 千円/人 / ベース 6,563.38 千円/人</t>
+          <t xml:space="preserve">補助 6,408.27 千円/人 / ベース 6,563.38 千円/人</t>
         </is>
       </c>
       <c r="J37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 6,694.92 千円/人 / ベース 6,712.9 千円/人</t>
+          <t xml:space="preserve">補助 6,583.33 千円/人 / ベース 6,712.9 千円/人</t>
         </is>
       </c>
       <c r="K37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 7,219.08 千円/人 / ベース 6,880.23 千円/人</t>
+          <t xml:space="preserve">補助 7,156.35 千円/人 / ベース 6,880.23 千円/人</t>
         </is>
       </c>
       <c r="L37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助 7,852.39 千円/人 / ベース 7,023.19 千円/人</t>
+          <t xml:space="preserve">補助 7,852.13 千円/人 / ベース 7,023.19 千円/人</t>
         </is>
       </c>
     </row>
@@ -5771,12 +5771,12 @@
       </c>
       <c r="K38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 89.36 %</t>
+          <t xml:space="preserve">寄与率 88.99 %</t>
         </is>
       </c>
       <c r="L38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">寄与率 90.94 %</t>
+          <t xml:space="preserve">寄与率 90.64 %</t>
         </is>
       </c>
     </row>
@@ -5786,7 +5786,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="68" customWidth="1"/>
@@ -5920,61 +5920,53 @@
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 従業員給与総額に占める給与の割合</t>
+          <t xml:space="preserve">補助事業 原価率（設備導入期間）</t>
         </is>
       </c>
       <c r="B6" s="2">
-        <v>95</v>
+        <v>68</v>
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D6" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E6" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="D6" s="2">
+        <v>68</v>
+      </c>
+      <c r="E6" s="2">
+        <v>68</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 従業員給与総額に占める給与の割合</t>
+          <t xml:space="preserve">ベース事業 原価率（設備導入期間）</t>
         </is>
       </c>
       <c r="B7" s="2">
-        <v>95</v>
+        <v>68</v>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D7" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E7" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="D7" s="2">
+        <v>68</v>
+      </c>
+      <c r="E7" s="2">
+        <v>68</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 役員給与総額に占める役員報酬の割合</t>
+          <t xml:space="preserve">補助事業 従業員給与総額に占める給与の割合</t>
         </is>
       </c>
       <c r="B8" s="2">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
@@ -5995,11 +5987,11 @@
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 役員給与総額に占める役員報酬の割合</t>
+          <t xml:space="preserve">ベース事業 従業員給与総額に占める給与の割合</t>
         </is>
       </c>
       <c r="B9" s="2">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C9" s="0" t="inlineStr">
         <is>
@@ -6020,11 +6012,11 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 研究開発費の売上高比率</t>
+          <t xml:space="preserve">補助事業 役員給与総額に占める役員報酬の割合</t>
         </is>
       </c>
       <c r="B10" s="2">
-        <v>0.5</v>
+        <v>90</v>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
@@ -6045,11 +6037,11 @@
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 研究開発費の売上高比率</t>
+          <t xml:space="preserve">ベース事業 役員給与総額に占める役員報酬の割合</t>
         </is>
       </c>
       <c r="B11" s="2">
-        <v>0.4</v>
+        <v>90</v>
       </c>
       <c r="C11" s="0" t="inlineStr">
         <is>
@@ -6070,11 +6062,11 @@
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 営業外損益の売上高比率</t>
+          <t xml:space="preserve">補助事業 研究開発費の売上高比率</t>
         </is>
       </c>
       <c r="B12" s="2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C12" s="0" t="inlineStr">
         <is>
@@ -6095,11 +6087,11 @@
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 営業外損益の売上高比率</t>
+          <t xml:space="preserve">ベース事業 研究開発費の売上高比率</t>
         </is>
       </c>
       <c r="B13" s="2">
-        <v>-0.5</v>
+        <v>0.4</v>
       </c>
       <c r="C13" s="0" t="inlineStr">
         <is>
@@ -6120,7 +6112,7 @@
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 特別損益の売上高比率</t>
+          <t xml:space="preserve">補助事業 営業外損益の売上高比率</t>
         </is>
       </c>
       <c r="B14" s="2">
@@ -6145,11 +6137,11 @@
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 特別損益の売上高比率</t>
+          <t xml:space="preserve">ベース事業 営業外損益の売上高比率</t>
         </is>
       </c>
       <c r="B15" s="2">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="C15" s="0" t="inlineStr">
         <is>
@@ -6170,11 +6162,11 @@
     <row r="16">
       <c r="A16" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">実効税率（当期純利益割合＝100%－実効税率）</t>
+          <t xml:space="preserve">補助事業 特別損益の売上高比率</t>
         </is>
       </c>
       <c r="B16" s="2">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
@@ -6195,32 +6187,36 @@
     <row r="17">
       <c r="A17" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 売上成長率（設備導入期間）</t>
+          <t xml:space="preserve">ベース事業 特別損益の売上高比率</t>
         </is>
       </c>
       <c r="B17" s="2">
-        <v>5.409356725146197</v>
+        <v>0</v>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D17" s="2">
-        <v>5.116959064327475</v>
-      </c>
-      <c r="E17" s="2">
-        <v>5.701754385964919</v>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E17" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 売上高（設備導入初年度）</t>
+          <t xml:space="preserve">実効税率（当期純利益割合＝100%－実効税率）</t>
         </is>
       </c>
       <c r="B18" s="2">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
@@ -6241,78 +6237,82 @@
     <row r="19">
       <c r="A19" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 売上高（基準年度）</t>
+          <t xml:space="preserve">補助事業 売上成長率（設備導入期間）</t>
         </is>
       </c>
       <c r="B19" s="2">
-        <v>0</v>
+        <v>5.409356725146197</v>
       </c>
       <c r="C19" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D19" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E19" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="D19" s="2">
+        <v>5.116959064327475</v>
+      </c>
+      <c r="E19" s="2">
+        <v>5.701754385964919</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 原価率改善ポイント（設備導入期間）</t>
+          <t xml:space="preserve">補助事業 売上高（設備導入初年度）</t>
         </is>
       </c>
       <c r="B20" s="2">
-        <v>5.551115123125783e-15</v>
+        <v>0</v>
       </c>
       <c r="C20" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D20" s="2">
-        <v>0</v>
-      </c>
-      <c r="E20" s="2">
-        <v>1.6653345369377348e-14</v>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E20" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 1人当たり給与支給総額上昇率（設備導入期間）</t>
+          <t xml:space="preserve">補助事業 売上高（基準年度）</t>
         </is>
       </c>
       <c r="B21" s="2">
-        <v>2.0030662342518046</v>
+        <v>0</v>
       </c>
       <c r="C21" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">基準年度額が最新決算期額以上（成長率0%以上）</t>
-        </is>
-      </c>
-      <c r="D21" s="2">
-        <v>1.9325330501846927</v>
-      </c>
-      <c r="E21" s="2">
-        <v>2.0735994183189166</v>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E21" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 常時使用する従業員数の成長率（設備導入期間）</t>
+          <t xml:space="preserve">補助事業 原価率改善ポイント（設備導入期間）</t>
         </is>
       </c>
       <c r="B22" s="2">
-        <v>5.409356725146197</v>
+        <v>5.551115123125783e-15</v>
       </c>
       <c r="C22" s="0" t="inlineStr">
         <is>
@@ -6320,37 +6320,37 @@
         </is>
       </c>
       <c r="D22" s="2">
-        <v>5.116959064327475</v>
+        <v>0</v>
       </c>
       <c r="E22" s="2">
-        <v>5.701754385964919</v>
+        <v>1.6653345369377348e-14</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 その他販管費率改善ポイント（設備導入期間）</t>
+          <t xml:space="preserve">補助事業 1人当たり給与支給総額上昇率（設備導入期間）</t>
         </is>
       </c>
       <c r="B23" s="2">
-        <v>0</v>
+        <v>2.0030662342518046</v>
       </c>
       <c r="C23" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">—</t>
+          <t xml:space="preserve">基準年度額が最新決算期額以上（成長率0%以上）</t>
         </is>
       </c>
       <c r="D23" s="2">
-        <v>0</v>
+        <v>1.9325330501846927</v>
       </c>
       <c r="E23" s="2">
-        <v>0</v>
+        <v>2.0735994183189166</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">役員1人当たり給与支給総額上昇率（設備導入期間）</t>
+          <t xml:space="preserve">補助事業 常時使用する従業員数の成長率（設備導入期間）</t>
         </is>
       </c>
       <c r="B24" s="2">
@@ -6371,11 +6371,11 @@
     <row r="25">
       <c r="A25" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 売上成長率（設備導入期間）</t>
+          <t xml:space="preserve">補助事業 その他販管費率改善ポイント（設備導入期間）</t>
         </is>
       </c>
       <c r="B25" s="2">
-        <v>4.257246376811585</v>
+        <v>0</v>
       </c>
       <c r="C25" s="0" t="inlineStr">
         <is>
@@ -6383,20 +6383,20 @@
         </is>
       </c>
       <c r="D25" s="2">
-        <v>4.076086956521719</v>
+        <v>0</v>
       </c>
       <c r="E25" s="2">
-        <v>4.438405797101453</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 原価率改善ポイント（設備導入期間）</t>
+          <t xml:space="preserve">役員1人当たり給与支給総額上昇率（設備導入期間）</t>
         </is>
       </c>
       <c r="B26" s="2">
-        <v>0</v>
+        <v>5.409356725146197</v>
       </c>
       <c r="C26" s="0" t="inlineStr">
         <is>
@@ -6404,20 +6404,20 @@
         </is>
       </c>
       <c r="D26" s="2">
-        <v>0</v>
+        <v>5.116959064327475</v>
       </c>
       <c r="E26" s="2">
-        <v>0.013457556935819737</v>
+        <v>5.701754385964919</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業1人当たり給与支給総額の年平均上昇率（設備導入期間）</t>
+          <t xml:space="preserve">ベース事業 売上成長率（設備導入期間）</t>
         </is>
       </c>
       <c r="B27" s="2">
-        <v>1.984645846924027</v>
+        <v>4.257246376811585</v>
       </c>
       <c r="C27" s="0" t="inlineStr">
         <is>
@@ -6425,45 +6425,41 @@
         </is>
       </c>
       <c r="D27" s="2">
-        <v>1.9139457023717443</v>
+        <v>4.076086956521719</v>
       </c>
       <c r="E27" s="2">
-        <v>2.0553459914763095</v>
+        <v>4.438405797101453</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 役員1人当たり給与支給総額上昇率（設備導入期間）</t>
+          <t xml:space="preserve">ベース事業 原価率改善ポイント（設備導入期間）</t>
         </is>
       </c>
       <c r="B28" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C28" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D28" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E28" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="D28" s="2">
+        <v>0</v>
+      </c>
+      <c r="E28" s="2">
+        <v>0.013457556935819737</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 常時使用する従業員数の成長率（設備導入期間）</t>
+          <t xml:space="preserve">ベース事業1人当たり給与支給総額の年平均上昇率（設備導入期間）</t>
         </is>
       </c>
       <c r="B29" s="2">
-        <v>4.083333333333339</v>
+        <v>1.984645846924027</v>
       </c>
       <c r="C29" s="0" t="inlineStr">
         <is>
@@ -6471,41 +6467,45 @@
         </is>
       </c>
       <c r="D29" s="2">
-        <v>3.9166666666666683</v>
+        <v>1.9139457023717443</v>
       </c>
       <c r="E29" s="2">
-        <v>4.250000000000009</v>
+        <v>2.0553459914763095</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 その他販管費率改善ポイント（設備導入期間）</t>
+          <t xml:space="preserve">ベース事業 役員1人当たり給与支給総額上昇率（設備導入期間）</t>
         </is>
       </c>
       <c r="B30" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C30" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D30" s="2">
-        <v>0</v>
-      </c>
-      <c r="E30" s="2">
-        <v>0</v>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E30" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 売上成長率（基準年度後）</t>
+          <t xml:space="preserve">ベース事業 常時使用する従業員数の成長率（設備導入期間）</t>
         </is>
       </c>
       <c r="B31" s="2">
-        <v>22</v>
+        <v>4.083333333333339</v>
       </c>
       <c r="C31" s="0" t="inlineStr">
         <is>
@@ -6513,20 +6513,20 @@
         </is>
       </c>
       <c r="D31" s="2">
-        <v>15</v>
+        <v>3.9166666666666683</v>
       </c>
       <c r="E31" s="2">
-        <v>30</v>
+        <v>4.250000000000009</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 売上成長率（基準年度後）</t>
+          <t xml:space="preserve">ベース事業 その他販管費率改善ポイント（設備導入期間）</t>
         </is>
       </c>
       <c r="B32" s="2">
-        <v>6.257246376811586</v>
+        <v>0</v>
       </c>
       <c r="C32" s="0" t="inlineStr">
         <is>
@@ -6534,20 +6534,20 @@
         </is>
       </c>
       <c r="D32" s="2">
-        <v>6.076086956521719</v>
+        <v>0</v>
       </c>
       <c r="E32" s="2">
-        <v>6.438405797101453</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 原価率改善ポイント（基準年度後）</t>
+          <t xml:space="preserve">補助事業 売上成長率（基準年度後）</t>
         </is>
       </c>
       <c r="B33" s="2">
-        <v>1.5</v>
+        <v>22</v>
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
@@ -6555,20 +6555,20 @@
         </is>
       </c>
       <c r="D33" s="2">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="E33" s="2">
-        <v>3</v>
+        <v>30</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 原価率改善ポイント（基準年度後）</t>
+          <t xml:space="preserve">ベース事業 売上成長率（基準年度後）</t>
         </is>
       </c>
       <c r="B34" s="2">
-        <v>0.5</v>
+        <v>6.257246376811586</v>
       </c>
       <c r="C34" s="0" t="inlineStr">
         <is>
@@ -6576,20 +6576,20 @@
         </is>
       </c>
       <c r="D34" s="2">
-        <v>0.5</v>
+        <v>6.076086956521719</v>
       </c>
       <c r="E34" s="2">
-        <v>0.5134575569358197</v>
+        <v>6.438405797101453</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業1人当たり給与支給総額の年平均上昇率</t>
+          <t xml:space="preserve">補助事業 原価率改善ポイント（基準年度後）</t>
         </is>
       </c>
       <c r="B35" s="2">
-        <v>7.000000000000001</v>
+        <v>1.5</v>
       </c>
       <c r="C35" s="0" t="inlineStr">
         <is>
@@ -6597,20 +6597,20 @@
         </is>
       </c>
       <c r="D35" s="2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E35" s="2">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業1人当たり給与支給総額の年平均上昇率（基準年度後）</t>
+          <t xml:space="preserve">ベース事業 原価率改善ポイント（基準年度後）</t>
         </is>
       </c>
       <c r="B36" s="2">
-        <v>2.484645846924027</v>
+        <v>0.5</v>
       </c>
       <c r="C36" s="0" t="inlineStr">
         <is>
@@ -6618,45 +6618,41 @@
         </is>
       </c>
       <c r="D36" s="2">
-        <v>2.4139457023717443</v>
+        <v>0.5</v>
       </c>
       <c r="E36" s="2">
-        <v>2.5553459914763095</v>
+        <v>0.5134575569358197</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 役員1人当たり給与支給総額上昇率（基準年度後）</t>
+          <t xml:space="preserve">補助事業1人当たり給与支給総額の年平均上昇率</t>
         </is>
       </c>
       <c r="B37" s="2">
-        <v>4.5</v>
+        <v>7.000000000000001</v>
       </c>
       <c r="C37" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D37" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E37" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="D37" s="2">
+        <v>5</v>
+      </c>
+      <c r="E37" s="2">
+        <v>10</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 常時使用する従業員数の成長率</t>
+          <t xml:space="preserve">ベース事業1人当たり給与支給総額の年平均上昇率（基準年度後）</t>
         </is>
       </c>
       <c r="B38" s="2">
-        <v>4</v>
+        <v>2.484645846924027</v>
       </c>
       <c r="C38" s="0" t="inlineStr">
         <is>
@@ -6664,41 +6660,45 @@
         </is>
       </c>
       <c r="D38" s="2">
-        <v>0</v>
+        <v>2.4139457023717443</v>
       </c>
       <c r="E38" s="2">
-        <v>8</v>
+        <v>2.5553459914763095</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 常時使用する従業員数の成長率（基準年度後）</t>
+          <t xml:space="preserve">ベース事業 役員1人当たり給与支給総額上昇率（基準年度後）</t>
         </is>
       </c>
       <c r="B39" s="2">
-        <v>4.583333333333338</v>
+        <v>4.5</v>
       </c>
       <c r="C39" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D39" s="2">
-        <v>4.416666666666668</v>
-      </c>
-      <c r="E39" s="2">
-        <v>4.750000000000009</v>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E39" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業 その他販管費率改善ポイント（基準年後）</t>
+          <t xml:space="preserve">補助事業 常時使用する従業員数の成長率</t>
         </is>
       </c>
       <c r="B40" s="2">
-        <v>1.5</v>
+        <v>4</v>
       </c>
       <c r="C40" s="0" t="inlineStr">
         <is>
@@ -6709,17 +6709,17 @@
         <v>0</v>
       </c>
       <c r="E40" s="2">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">ベース事業 その他販管費率改善ポイント（基準年後）</t>
+          <t xml:space="preserve">ベース事業 常時使用する従業員数の成長率（基準年度後）</t>
         </is>
       </c>
       <c r="B41" s="2">
-        <v>0.5</v>
+        <v>4.583333333333338</v>
       </c>
       <c r="C41" s="0" t="inlineStr">
         <is>
@@ -6727,20 +6727,20 @@
         </is>
       </c>
       <c r="D41" s="2">
-        <v>0</v>
+        <v>4.416666666666668</v>
       </c>
       <c r="E41" s="2">
-        <v>1</v>
+        <v>4.750000000000009</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">役員1人当たり給与支給総額の年平均上昇率</t>
+          <t xml:space="preserve">補助事業 その他販管費率改善ポイント（基準年後）</t>
         </is>
       </c>
       <c r="B42" s="2">
-        <v>5.380116959064325</v>
+        <v>1.5</v>
       </c>
       <c r="C42" s="0" t="inlineStr">
         <is>
@@ -6748,57 +6748,99 @@
         </is>
       </c>
       <c r="D42" s="2">
-        <v>4.263157894736836</v>
+        <v>0</v>
       </c>
       <c r="E42" s="2">
-        <v>6.555555555555557</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">補助事業投資額</t>
+          <t xml:space="preserve">ベース事業 その他販管費率改善ポイント（基準年後）</t>
         </is>
       </c>
       <c r="B43" s="2">
-        <v>2300000</v>
+        <v>0.5</v>
       </c>
       <c r="C43" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">20億円以上（専門家経費・外注費を除く補助対象経費）</t>
-        </is>
-      </c>
-      <c r="D43" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E43" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D43" s="2">
+        <v>0</v>
+      </c>
+      <c r="E43" s="2">
+        <v>1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">役員1人当たり給与支給総額の年平均上昇率</t>
+        </is>
+      </c>
+      <c r="B44" s="2">
+        <v>5.380116959064325</v>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D44" s="2">
+        <v>4.263157894736836</v>
+      </c>
+      <c r="E44" s="2">
+        <v>6.555555555555557</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">補助事業投資額</t>
+        </is>
+      </c>
+      <c r="B45" s="2">
+        <v>2300000</v>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20億円以上（専門家経費・外注費を除く補助対象経費）</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">申請補助金額</t>
         </is>
       </c>
-      <c r="B44" s="2">
+      <c r="B46" s="2">
         <v>766000</v>
       </c>
-      <c r="C44" s="0" t="inlineStr">
+      <c r="C46" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">50億円以下、かつ投資額の1/3以下（現在上限7.67億円）</t>
         </is>
       </c>
-      <c r="D44" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E44" s="0" t="inlineStr">
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E46" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -6810,7 +6852,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C295"/>
+  <dimension ref="A1:C301"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="72" customWidth="1"/>
@@ -8970,11 +9012,11 @@
     <row r="144">
       <c r="A144" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherCogsRateWhenSalesZero:0</t>
+          <t xml:space="preserve">driver-range:otherCogsRateToBase:0</t>
         </is>
       </c>
       <c r="B144" s="2">
-        <v>0.66</v>
+        <v>0.68</v>
       </c>
       <c r="C144" s="0" t="inlineStr">
         <is>
@@ -8985,11 +9027,11 @@
     <row r="145">
       <c r="A145" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherCogsRateWhenSalesZero:1</t>
+          <t xml:space="preserve">driver-range:otherCogsRateToBase:1</t>
         </is>
       </c>
       <c r="B145" s="2">
-        <v>0.7</v>
+        <v>0.68</v>
       </c>
       <c r="C145" s="0" t="inlineStr">
         <is>
@@ -9000,26 +9042,26 @@
     <row r="146">
       <c r="A146" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherEmployeeSalaryShare:0</t>
+          <t xml:space="preserve">driver-range:otherCogsRateWhenSalesZero:0</t>
         </is>
       </c>
       <c r="B146" s="2">
-        <v>0</v>
+        <v>0.66</v>
       </c>
       <c r="C146" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherEmployeeSalaryShare:1</t>
+          <t xml:space="preserve">driver-range:otherCogsRateWhenSalesZero:1</t>
         </is>
       </c>
       <c r="B147" s="2">
-        <v>1</v>
+        <v>0.7</v>
       </c>
       <c r="C147" s="0" t="inlineStr">
         <is>
@@ -9030,26 +9072,26 @@
     <row r="148">
       <c r="A148" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherExtraordinaryRate:0</t>
+          <t xml:space="preserve">driver-range:otherEmployeeSalaryShare:0</t>
         </is>
       </c>
       <c r="B148" s="2">
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="C148" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherExtraordinaryRate:1</t>
+          <t xml:space="preserve">driver-range:otherEmployeeSalaryShare:1</t>
         </is>
       </c>
       <c r="B149" s="2">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="C149" s="0" t="inlineStr">
         <is>
@@ -9060,11 +9102,11 @@
     <row r="150">
       <c r="A150" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherHeadcountGrowth:0</t>
+          <t xml:space="preserve">driver-range:otherExtraordinaryRate:0</t>
         </is>
       </c>
       <c r="B150" s="2">
-        <v>0.04416666666666668</v>
+        <v>-0.5</v>
       </c>
       <c r="C150" s="0" t="inlineStr">
         <is>
@@ -9075,11 +9117,11 @@
     <row r="151">
       <c r="A151" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherHeadcountGrowth:1</t>
+          <t xml:space="preserve">driver-range:otherExtraordinaryRate:1</t>
         </is>
       </c>
       <c r="B151" s="2">
-        <v>0.04750000000000009</v>
+        <v>0.5</v>
       </c>
       <c r="C151" s="0" t="inlineStr">
         <is>
@@ -9090,11 +9132,11 @@
     <row r="152">
       <c r="A152" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherHeadcountGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:otherHeadcountGrowth:0</t>
         </is>
       </c>
       <c r="B152" s="2">
-        <v>0.03916666666666668</v>
+        <v>0.04416666666666668</v>
       </c>
       <c r="C152" s="0" t="inlineStr">
         <is>
@@ -9105,11 +9147,11 @@
     <row r="153">
       <c r="A153" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherHeadcountGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:otherHeadcountGrowth:1</t>
         </is>
       </c>
       <c r="B153" s="2">
-        <v>0.04250000000000009</v>
+        <v>0.04750000000000009</v>
       </c>
       <c r="C153" s="0" t="inlineStr">
         <is>
@@ -9120,11 +9162,11 @@
     <row r="154">
       <c r="A154" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherNonOperatingRate:0</t>
+          <t xml:space="preserve">driver-range:otherHeadcountGrowthToBase:0</t>
         </is>
       </c>
       <c r="B154" s="2">
-        <v>-0.5</v>
+        <v>0.03916666666666668</v>
       </c>
       <c r="C154" s="0" t="inlineStr">
         <is>
@@ -9135,11 +9177,11 @@
     <row r="155">
       <c r="A155" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherNonOperatingRate:1</t>
+          <t xml:space="preserve">driver-range:otherHeadcountGrowthToBase:1</t>
         </is>
       </c>
       <c r="B155" s="2">
-        <v>0.5</v>
+        <v>0.04250000000000009</v>
       </c>
       <c r="C155" s="0" t="inlineStr">
         <is>
@@ -9150,26 +9192,26 @@
     <row r="156">
       <c r="A156" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherOfficerCompensationShare:0</t>
+          <t xml:space="preserve">driver-range:otherNonOperatingRate:0</t>
         </is>
       </c>
       <c r="B156" s="2">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="C156" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherOfficerCompensationShare:1</t>
+          <t xml:space="preserve">driver-range:otherNonOperatingRate:1</t>
         </is>
       </c>
       <c r="B157" s="2">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="C157" s="0" t="inlineStr">
         <is>
@@ -9180,7 +9222,7 @@
     <row r="158">
       <c r="A158" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherOfficerPayGrowth:0</t>
+          <t xml:space="preserve">driver-range:otherOfficerCompensationShare:0</t>
         </is>
       </c>
       <c r="B158" s="2">
@@ -9195,11 +9237,11 @@
     <row r="159">
       <c r="A159" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherOfficerPayGrowth:1</t>
+          <t xml:space="preserve">driver-range:otherOfficerCompensationShare:1</t>
         </is>
       </c>
       <c r="B159" s="2">
-        <v>0.08</v>
+        <v>1</v>
       </c>
       <c r="C159" s="0" t="inlineStr">
         <is>
@@ -9210,7 +9252,7 @@
     <row r="160">
       <c r="A160" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherOfficerPayGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:otherOfficerPayGrowth:0</t>
         </is>
       </c>
       <c r="B160" s="2">
@@ -9225,7 +9267,7 @@
     <row r="161">
       <c r="A161" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherOfficerPayGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:otherOfficerPayGrowth:1</t>
         </is>
       </c>
       <c r="B161" s="2">
@@ -9240,26 +9282,26 @@
     <row r="162">
       <c r="A162" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherPayGrowth:0</t>
+          <t xml:space="preserve">driver-range:otherOfficerPayGrowthToBase:0</t>
         </is>
       </c>
       <c r="B162" s="2">
-        <v>0.024139457023717444</v>
+        <v>0</v>
       </c>
       <c r="C162" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherPayGrowth:1</t>
+          <t xml:space="preserve">driver-range:otherOfficerPayGrowthToBase:1</t>
         </is>
       </c>
       <c r="B163" s="2">
-        <v>0.025553459914763096</v>
+        <v>0.08</v>
       </c>
       <c r="C163" s="0" t="inlineStr">
         <is>
@@ -9270,11 +9312,11 @@
     <row r="164">
       <c r="A164" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherPayGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:otherPayGrowth:0</t>
         </is>
       </c>
       <c r="B164" s="2">
-        <v>0.019139457023717443</v>
+        <v>0.024139457023717444</v>
       </c>
       <c r="C164" s="0" t="inlineStr">
         <is>
@@ -9285,11 +9327,11 @@
     <row r="165">
       <c r="A165" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherPayGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:otherPayGrowth:1</t>
         </is>
       </c>
       <c r="B165" s="2">
-        <v>0.020553459914763095</v>
+        <v>0.025553459914763096</v>
       </c>
       <c r="C165" s="0" t="inlineStr">
         <is>
@@ -9300,26 +9342,26 @@
     <row r="166">
       <c r="A166" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherResearchDevelopmentRate:0</t>
+          <t xml:space="preserve">driver-range:otherPayGrowthToBase:0</t>
         </is>
       </c>
       <c r="B166" s="2">
-        <v>0</v>
+        <v>0.019139457023717443</v>
       </c>
       <c r="C166" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherResearchDevelopmentRate:1</t>
+          <t xml:space="preserve">driver-range:otherPayGrowthToBase:1</t>
         </is>
       </c>
       <c r="B167" s="2">
-        <v>0.3</v>
+        <v>0.020553459914763095</v>
       </c>
       <c r="C167" s="0" t="inlineStr">
         <is>
@@ -9330,26 +9372,26 @@
     <row r="168">
       <c r="A168" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSalesGrowth:0</t>
+          <t xml:space="preserve">driver-range:otherResearchDevelopmentRate:0</t>
         </is>
       </c>
       <c r="B168" s="2">
-        <v>0.06076086956521719</v>
+        <v>0</v>
       </c>
       <c r="C168" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSalesGrowth:1</t>
+          <t xml:space="preserve">driver-range:otherResearchDevelopmentRate:1</t>
         </is>
       </c>
       <c r="B169" s="2">
-        <v>0.06438405797101453</v>
+        <v>0.3</v>
       </c>
       <c r="C169" s="0" t="inlineStr">
         <is>
@@ -9360,11 +9402,11 @@
     <row r="170">
       <c r="A170" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSalesGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:otherSalesGrowth:0</t>
         </is>
       </c>
       <c r="B170" s="2">
-        <v>0.040760869565217184</v>
+        <v>0.06076086956521719</v>
       </c>
       <c r="C170" s="0" t="inlineStr">
         <is>
@@ -9375,11 +9417,11 @@
     <row r="171">
       <c r="A171" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSalesGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:otherSalesGrowth:1</t>
         </is>
       </c>
       <c r="B171" s="2">
-        <v>0.04438405797101452</v>
+        <v>0.06438405797101453</v>
       </c>
       <c r="C171" s="0" t="inlineStr">
         <is>
@@ -9390,37 +9432,37 @@
     <row r="172">
       <c r="A172" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSgaImprovementToBase:0</t>
+          <t xml:space="preserve">driver-range:otherSalesGrowthToBase:0</t>
         </is>
       </c>
       <c r="B172" s="2">
-        <v>0</v>
+        <v>0.040760869565217184</v>
       </c>
       <c r="C172" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSgaImprovementToBase:1</t>
+          <t xml:space="preserve">driver-range:otherSalesGrowthToBase:1</t>
         </is>
       </c>
       <c r="B173" s="2">
-        <v>0</v>
+        <v>0.04438405797101452</v>
       </c>
       <c r="C173" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSgaRateEnd:0</t>
+          <t xml:space="preserve">driver-range:otherSgaImprovementToBase:0</t>
         </is>
       </c>
       <c r="B174" s="2">
@@ -9435,22 +9477,22 @@
     <row r="175">
       <c r="A175" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:otherSgaRateEnd:1</t>
+          <t xml:space="preserve">driver-range:otherSgaImprovementToBase:1</t>
         </is>
       </c>
       <c r="B175" s="2">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="C175" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectBaseYearSales:0</t>
+          <t xml:space="preserve">driver-range:otherSgaRateEnd:0</t>
         </is>
       </c>
       <c r="B176" s="2">
@@ -9465,11 +9507,11 @@
     <row r="177">
       <c r="A177" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectBaseYearSales:1</t>
+          <t xml:space="preserve">driver-range:otherSgaRateEnd:1</t>
         </is>
       </c>
       <c r="B177" s="2">
-        <v>10000000000</v>
+        <v>0.01</v>
       </c>
       <c r="C177" s="0" t="inlineStr">
         <is>
@@ -9480,7 +9522,7 @@
     <row r="178">
       <c r="A178" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectCogsDepreciationShare:0</t>
+          <t xml:space="preserve">driver-range:projectBaseYearSales:0</t>
         </is>
       </c>
       <c r="B178" s="2">
@@ -9495,11 +9537,11 @@
     <row r="179">
       <c r="A179" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectCogsDepreciationShare:1</t>
+          <t xml:space="preserve">driver-range:projectBaseYearSales:1</t>
         </is>
       </c>
       <c r="B179" s="2">
-        <v>1</v>
+        <v>10000000000</v>
       </c>
       <c r="C179" s="0" t="inlineStr">
         <is>
@@ -9510,7 +9552,7 @@
     <row r="180">
       <c r="A180" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectCogsImprovementAfterBase:0</t>
+          <t xml:space="preserve">driver-range:projectCogsDepreciationShare:0</t>
         </is>
       </c>
       <c r="B180" s="2">
@@ -9525,11 +9567,11 @@
     <row r="181">
       <c r="A181" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectCogsImprovementAfterBase:1</t>
+          <t xml:space="preserve">driver-range:projectCogsDepreciationShare:1</t>
         </is>
       </c>
       <c r="B181" s="2">
-        <v>0.03</v>
+        <v>1</v>
       </c>
       <c r="C181" s="0" t="inlineStr">
         <is>
@@ -9540,7 +9582,7 @@
     <row r="182">
       <c r="A182" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectCogsImprovementToBase:0</t>
+          <t xml:space="preserve">driver-range:projectCogsImprovementAfterBase:0</t>
         </is>
       </c>
       <c r="B182" s="2">
@@ -9555,11 +9597,11 @@
     <row r="183">
       <c r="A183" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectCogsImprovementToBase:1</t>
+          <t xml:space="preserve">driver-range:projectCogsImprovementAfterBase:1</t>
         </is>
       </c>
       <c r="B183" s="2">
-        <v>1.6653345369377348e-16</v>
+        <v>0.03</v>
       </c>
       <c r="C183" s="0" t="inlineStr">
         <is>
@@ -9570,26 +9612,26 @@
     <row r="184">
       <c r="A184" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectCogsRateWhenSalesZero:0</t>
+          <t xml:space="preserve">driver-range:projectCogsImprovementToBase:0</t>
         </is>
       </c>
       <c r="B184" s="2">
-        <v>0.66</v>
+        <v>0</v>
       </c>
       <c r="C184" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectCogsRateWhenSalesZero:1</t>
+          <t xml:space="preserve">driver-range:projectCogsImprovementToBase:1</t>
         </is>
       </c>
       <c r="B185" s="2">
-        <v>0.7</v>
+        <v>1.6653345369377348e-16</v>
       </c>
       <c r="C185" s="0" t="inlineStr">
         <is>
@@ -9600,26 +9642,26 @@
     <row r="186">
       <c r="A186" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectEmployeeSalaryShare:0</t>
+          <t xml:space="preserve">driver-range:projectCogsRateToBase:0</t>
         </is>
       </c>
       <c r="B186" s="2">
-        <v>0</v>
+        <v>0.68</v>
       </c>
       <c r="C186" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectEmployeeSalaryShare:1</t>
+          <t xml:space="preserve">driver-range:projectCogsRateToBase:1</t>
         </is>
       </c>
       <c r="B187" s="2">
-        <v>1</v>
+        <v>0.68</v>
       </c>
       <c r="C187" s="0" t="inlineStr">
         <is>
@@ -9630,11 +9672,11 @@
     <row r="188">
       <c r="A188" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectExtraordinaryRate:0</t>
+          <t xml:space="preserve">driver-range:projectCogsRateWhenSalesZero:0</t>
         </is>
       </c>
       <c r="B188" s="2">
-        <v>-0.5</v>
+        <v>0.66</v>
       </c>
       <c r="C188" s="0" t="inlineStr">
         <is>
@@ -9645,11 +9687,11 @@
     <row r="189">
       <c r="A189" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectExtraordinaryRate:1</t>
+          <t xml:space="preserve">driver-range:projectCogsRateWhenSalesZero:1</t>
         </is>
       </c>
       <c r="B189" s="2">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="C189" s="0" t="inlineStr">
         <is>
@@ -9660,7 +9702,7 @@
     <row r="190">
       <c r="A190" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectFirstYearSales:0</t>
+          <t xml:space="preserve">driver-range:projectEmployeeSalaryShare:0</t>
         </is>
       </c>
       <c r="B190" s="2">
@@ -9675,11 +9717,11 @@
     <row r="191">
       <c r="A191" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectFirstYearSales:1</t>
+          <t xml:space="preserve">driver-range:projectEmployeeSalaryShare:1</t>
         </is>
       </c>
       <c r="B191" s="2">
-        <v>10000000000</v>
+        <v>1</v>
       </c>
       <c r="C191" s="0" t="inlineStr">
         <is>
@@ -9690,26 +9732,26 @@
     <row r="192">
       <c r="A192" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectHeadcountGrowth:0</t>
+          <t xml:space="preserve">driver-range:projectExtraordinaryRate:0</t>
         </is>
       </c>
       <c r="B192" s="2">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="C192" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectHeadcountGrowth:1</t>
+          <t xml:space="preserve">driver-range:projectExtraordinaryRate:1</t>
         </is>
       </c>
       <c r="B193" s="2">
-        <v>0.08</v>
+        <v>0.5</v>
       </c>
       <c r="C193" s="0" t="inlineStr">
         <is>
@@ -9720,26 +9762,26 @@
     <row r="194">
       <c r="A194" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectHeadcountGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:projectFirstYearSales:0</t>
         </is>
       </c>
       <c r="B194" s="2">
-        <v>0.051169590643274754</v>
+        <v>0</v>
       </c>
       <c r="C194" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectHeadcountGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:projectFirstYearSales:1</t>
         </is>
       </c>
       <c r="B195" s="2">
-        <v>0.05701754385964919</v>
+        <v>10000000000</v>
       </c>
       <c r="C195" s="0" t="inlineStr">
         <is>
@@ -9750,26 +9792,26 @@
     <row r="196">
       <c r="A196" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectMarketGrowth:0</t>
+          <t xml:space="preserve">driver-range:projectHeadcountGrowth:0</t>
         </is>
       </c>
       <c r="B196" s="2">
-        <v>-0.05</v>
+        <v>0</v>
       </c>
       <c r="C196" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectMarketGrowth:1</t>
+          <t xml:space="preserve">driver-range:projectHeadcountGrowth:1</t>
         </is>
       </c>
       <c r="B197" s="2">
-        <v>0.3</v>
+        <v>0.08</v>
       </c>
       <c r="C197" s="0" t="inlineStr">
         <is>
@@ -9780,11 +9822,11 @@
     <row r="198">
       <c r="A198" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectNonOperatingRate:0</t>
+          <t xml:space="preserve">driver-range:projectHeadcountGrowthToBase:0</t>
         </is>
       </c>
       <c r="B198" s="2">
-        <v>-0.5</v>
+        <v>0.051169590643274754</v>
       </c>
       <c r="C198" s="0" t="inlineStr">
         <is>
@@ -9795,11 +9837,11 @@
     <row r="199">
       <c r="A199" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectNonOperatingRate:1</t>
+          <t xml:space="preserve">driver-range:projectHeadcountGrowthToBase:1</t>
         </is>
       </c>
       <c r="B199" s="2">
-        <v>0.5</v>
+        <v>0.05701754385964919</v>
       </c>
       <c r="C199" s="0" t="inlineStr">
         <is>
@@ -9810,26 +9852,26 @@
     <row r="200">
       <c r="A200" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectOfficerCompensationShare:0</t>
+          <t xml:space="preserve">driver-range:projectMarketGrowth:0</t>
         </is>
       </c>
       <c r="B200" s="2">
-        <v>0</v>
+        <v>-0.05</v>
       </c>
       <c r="C200" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectOfficerCompensationShare:1</t>
+          <t xml:space="preserve">driver-range:projectMarketGrowth:1</t>
         </is>
       </c>
       <c r="B201" s="2">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="C201" s="0" t="inlineStr">
         <is>
@@ -9840,11 +9882,11 @@
     <row r="202">
       <c r="A202" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectOfficerPayGrowth:0</t>
+          <t xml:space="preserve">driver-range:projectNonOperatingRate:0</t>
         </is>
       </c>
       <c r="B202" s="2">
-        <v>0.04263157894736836</v>
+        <v>-0.5</v>
       </c>
       <c r="C202" s="0" t="inlineStr">
         <is>
@@ -9855,11 +9897,11 @@
     <row r="203">
       <c r="A203" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectOfficerPayGrowth:1</t>
+          <t xml:space="preserve">driver-range:projectNonOperatingRate:1</t>
         </is>
       </c>
       <c r="B203" s="2">
-        <v>0.06555555555555558</v>
+        <v>0.5</v>
       </c>
       <c r="C203" s="0" t="inlineStr">
         <is>
@@ -9870,26 +9912,26 @@
     <row r="204">
       <c r="A204" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectOfficerPayGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:projectOfficerCompensationShare:0</t>
         </is>
       </c>
       <c r="B204" s="2">
-        <v>0.051169590643274754</v>
+        <v>0</v>
       </c>
       <c r="C204" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectOfficerPayGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:projectOfficerCompensationShare:1</t>
         </is>
       </c>
       <c r="B205" s="2">
-        <v>0.05701754385964919</v>
+        <v>1</v>
       </c>
       <c r="C205" s="0" t="inlineStr">
         <is>
@@ -9900,11 +9942,11 @@
     <row r="206">
       <c r="A206" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectPayGrowth:0</t>
+          <t xml:space="preserve">driver-range:projectOfficerPayGrowth:0</t>
         </is>
       </c>
       <c r="B206" s="2">
-        <v>0.05</v>
+        <v>0.04263157894736836</v>
       </c>
       <c r="C206" s="0" t="inlineStr">
         <is>
@@ -9915,11 +9957,11 @@
     <row r="207">
       <c r="A207" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectPayGrowth:1</t>
+          <t xml:space="preserve">driver-range:projectOfficerPayGrowth:1</t>
         </is>
       </c>
       <c r="B207" s="2">
-        <v>0.1</v>
+        <v>0.06555555555555558</v>
       </c>
       <c r="C207" s="0" t="inlineStr">
         <is>
@@ -9930,11 +9972,11 @@
     <row r="208">
       <c r="A208" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectPayGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:projectOfficerPayGrowthToBase:0</t>
         </is>
       </c>
       <c r="B208" s="2">
-        <v>0.019325330501846927</v>
+        <v>0.051169590643274754</v>
       </c>
       <c r="C208" s="0" t="inlineStr">
         <is>
@@ -9945,11 +9987,11 @@
     <row r="209">
       <c r="A209" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectPayGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:projectOfficerPayGrowthToBase:1</t>
         </is>
       </c>
       <c r="B209" s="2">
-        <v>0.020735994183189166</v>
+        <v>0.05701754385964919</v>
       </c>
       <c r="C209" s="0" t="inlineStr">
         <is>
@@ -9960,26 +10002,26 @@
     <row r="210">
       <c r="A210" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectResearchDevelopmentRate:0</t>
+          <t xml:space="preserve">driver-range:projectPayGrowth:0</t>
         </is>
       </c>
       <c r="B210" s="2">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="C210" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectResearchDevelopmentRate:1</t>
+          <t xml:space="preserve">driver-range:projectPayGrowth:1</t>
         </is>
       </c>
       <c r="B211" s="2">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="C211" s="0" t="inlineStr">
         <is>
@@ -9990,11 +10032,11 @@
     <row r="212">
       <c r="A212" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSalesGrowth:0</t>
+          <t xml:space="preserve">driver-range:projectPayGrowthToBase:0</t>
         </is>
       </c>
       <c r="B212" s="2">
-        <v>0.15</v>
+        <v>0.019325330501846927</v>
       </c>
       <c r="C212" s="0" t="inlineStr">
         <is>
@@ -10005,11 +10047,11 @@
     <row r="213">
       <c r="A213" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSalesGrowth:1</t>
+          <t xml:space="preserve">driver-range:projectPayGrowthToBase:1</t>
         </is>
       </c>
       <c r="B213" s="2">
-        <v>0.3</v>
+        <v>0.020735994183189166</v>
       </c>
       <c r="C213" s="0" t="inlineStr">
         <is>
@@ -10020,26 +10062,26 @@
     <row r="214">
       <c r="A214" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSalesGrowthToBase:0</t>
+          <t xml:space="preserve">driver-range:projectResearchDevelopmentRate:0</t>
         </is>
       </c>
       <c r="B214" s="2">
-        <v>0.051169590643274754</v>
+        <v>0</v>
       </c>
       <c r="C214" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSalesGrowthToBase:1</t>
+          <t xml:space="preserve">driver-range:projectResearchDevelopmentRate:1</t>
         </is>
       </c>
       <c r="B215" s="2">
-        <v>0.05701754385964919</v>
+        <v>0.3</v>
       </c>
       <c r="C215" s="0" t="inlineStr">
         <is>
@@ -10050,56 +10092,56 @@
     <row r="216">
       <c r="A216" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSgaImprovementToBase:0</t>
+          <t xml:space="preserve">driver-range:projectSalesGrowth:0</t>
         </is>
       </c>
       <c r="B216" s="2">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="C216" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSgaImprovementToBase:1</t>
+          <t xml:space="preserve">driver-range:projectSalesGrowth:1</t>
         </is>
       </c>
       <c r="B217" s="2">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="C217" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSgaRateEnd:0</t>
+          <t xml:space="preserve">driver-range:projectSalesGrowthToBase:0</t>
         </is>
       </c>
       <c r="B218" s="2">
-        <v>0</v>
+        <v>0.051169590643274754</v>
       </c>
       <c r="C218" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:projectSgaRateEnd:1</t>
+          <t xml:space="preserve">driver-range:projectSalesGrowthToBase:1</t>
         </is>
       </c>
       <c r="B219" s="2">
-        <v>0.03</v>
+        <v>0.05701754385964919</v>
       </c>
       <c r="C219" s="0" t="inlineStr">
         <is>
@@ -10110,56 +10152,56 @@
     <row r="220">
       <c r="A220" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:subsidy:0</t>
+          <t xml:space="preserve">driver-range:projectSgaImprovementToBase:0</t>
         </is>
       </c>
       <c r="B220" s="2">
-        <v>100000</v>
+        <v>0</v>
       </c>
       <c r="C220" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver-range:subsidy:1</t>
+          <t xml:space="preserve">driver-range:projectSgaImprovementToBase:1</t>
         </is>
       </c>
       <c r="B221" s="2">
-        <v>5000000</v>
+        <v>0</v>
       </c>
       <c r="C221" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:effectiveTaxRate</t>
+          <t xml:space="preserve">driver-range:projectSgaRateEnd:0</t>
         </is>
       </c>
       <c r="B222" s="2">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="C222" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:investment</t>
+          <t xml:space="preserve">driver-range:projectSgaRateEnd:1</t>
         </is>
       </c>
       <c r="B223" s="2">
-        <v>2300000</v>
+        <v>0.03</v>
       </c>
       <c r="C223" s="0" t="inlineStr">
         <is>
@@ -10170,11 +10212,11 @@
     <row r="224">
       <c r="A224" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:localBenchmark</t>
+          <t xml:space="preserve">driver-range:subsidy:0</t>
         </is>
       </c>
       <c r="B224" s="2">
-        <v>23</v>
+        <v>100000</v>
       </c>
       <c r="C224" s="0" t="inlineStr">
         <is>
@@ -10185,11 +10227,11 @@
     <row r="225">
       <c r="A225" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherCogsDepreciationShare</t>
+          <t xml:space="preserve">driver-range:subsidy:1</t>
         </is>
       </c>
       <c r="B225" s="2">
-        <v>0.2</v>
+        <v>5000000</v>
       </c>
       <c r="C225" s="0" t="inlineStr">
         <is>
@@ -10200,11 +10242,11 @@
     <row r="226">
       <c r="A226" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherCogsImprovement</t>
+          <t xml:space="preserve">driver:effectiveTaxRate</t>
         </is>
       </c>
       <c r="B226" s="2">
-        <v>0.005</v>
+        <v>0.3</v>
       </c>
       <c r="C226" s="0" t="inlineStr">
         <is>
@@ -10215,26 +10257,26 @@
     <row r="227">
       <c r="A227" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherCogsImprovementToBase</t>
+          <t xml:space="preserve">driver:investment</t>
         </is>
       </c>
       <c r="B227" s="2">
-        <v>0</v>
+        <v>2300000</v>
       </c>
       <c r="C227" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherCogsRateWhenSalesZero</t>
+          <t xml:space="preserve">driver:localBenchmark</t>
         </is>
       </c>
       <c r="B228" s="2">
-        <v>0.68</v>
+        <v>23</v>
       </c>
       <c r="C228" s="0" t="inlineStr">
         <is>
@@ -10245,11 +10287,11 @@
     <row r="229">
       <c r="A229" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherEmployeeSalaryShare</t>
+          <t xml:space="preserve">driver:otherCogsDepreciationShare</t>
         </is>
       </c>
       <c r="B229" s="2">
-        <v>0.95</v>
+        <v>0.2</v>
       </c>
       <c r="C229" s="0" t="inlineStr">
         <is>
@@ -10260,41 +10302,41 @@
     <row r="230">
       <c r="A230" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherExtraordinaryRate</t>
+          <t xml:space="preserve">driver:otherCogsImprovement</t>
         </is>
       </c>
       <c r="B230" s="2">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="C230" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherHeadcountGrowth</t>
+          <t xml:space="preserve">driver:otherCogsImprovementToBase</t>
         </is>
       </c>
       <c r="B231" s="2">
-        <v>0.045833333333333386</v>
+        <v>0</v>
       </c>
       <c r="C231" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherHeadcountGrowthToBase</t>
+          <t xml:space="preserve">driver:otherCogsRateToBase</t>
         </is>
       </c>
       <c r="B232" s="2">
-        <v>0.04083333333333339</v>
+        <v>0.68</v>
       </c>
       <c r="C232" s="0" t="inlineStr">
         <is>
@@ -10305,11 +10347,11 @@
     <row r="233">
       <c r="A233" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherNonOperatingRate</t>
+          <t xml:space="preserve">driver:otherCogsRateWhenSalesZero</t>
         </is>
       </c>
       <c r="B233" s="2">
-        <v>-0.005</v>
+        <v>0.68</v>
       </c>
       <c r="C233" s="0" t="inlineStr">
         <is>
@@ -10320,11 +10362,11 @@
     <row r="234">
       <c r="A234" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherOfficerCompensationShare</t>
+          <t xml:space="preserve">driver:otherEmployeeSalaryShare</t>
         </is>
       </c>
       <c r="B234" s="2">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="C234" s="0" t="inlineStr">
         <is>
@@ -10335,26 +10377,26 @@
     <row r="235">
       <c r="A235" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherOfficerPayGrowth</t>
+          <t xml:space="preserve">driver:otherExtraordinaryRate</t>
         </is>
       </c>
       <c r="B235" s="2">
-        <v>0.045</v>
+        <v>0</v>
       </c>
       <c r="C235" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherOfficerPayGrowthToBase</t>
+          <t xml:space="preserve">driver:otherHeadcountGrowth</t>
         </is>
       </c>
       <c r="B236" s="2">
-        <v>0.04</v>
+        <v>0.045833333333333386</v>
       </c>
       <c r="C236" s="0" t="inlineStr">
         <is>
@@ -10365,11 +10407,11 @@
     <row r="237">
       <c r="A237" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherPayGrowth</t>
+          <t xml:space="preserve">driver:otherHeadcountGrowthToBase</t>
         </is>
       </c>
       <c r="B237" s="2">
-        <v>0.02484645846924027</v>
+        <v>0.04083333333333339</v>
       </c>
       <c r="C237" s="0" t="inlineStr">
         <is>
@@ -10380,11 +10422,11 @@
     <row r="238">
       <c r="A238" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherPayGrowthToBase</t>
+          <t xml:space="preserve">driver:otherNonOperatingRate</t>
         </is>
       </c>
       <c r="B238" s="2">
-        <v>0.01984645846924027</v>
+        <v>-0.005</v>
       </c>
       <c r="C238" s="0" t="inlineStr">
         <is>
@@ -10395,11 +10437,11 @@
     <row r="239">
       <c r="A239" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherResearchDevelopmentRate</t>
+          <t xml:space="preserve">driver:otherOfficerCompensationShare</t>
         </is>
       </c>
       <c r="B239" s="2">
-        <v>0.004</v>
+        <v>0.9</v>
       </c>
       <c r="C239" s="0" t="inlineStr">
         <is>
@@ -10410,11 +10452,11 @@
     <row r="240">
       <c r="A240" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherSalesGrowth</t>
+          <t xml:space="preserve">driver:otherOfficerPayGrowth</t>
         </is>
       </c>
       <c r="B240" s="2">
-        <v>0.06257246376811586</v>
+        <v>0.045</v>
       </c>
       <c r="C240" s="0" t="inlineStr">
         <is>
@@ -10425,11 +10467,11 @@
     <row r="241">
       <c r="A241" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherSalesGrowthToBase</t>
+          <t xml:space="preserve">driver:otherOfficerPayGrowthToBase</t>
         </is>
       </c>
       <c r="B241" s="2">
-        <v>0.042572463768115854</v>
+        <v>0.04</v>
       </c>
       <c r="C241" s="0" t="inlineStr">
         <is>
@@ -10440,26 +10482,26 @@
     <row r="242">
       <c r="A242" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherSgaImprovementToBase</t>
+          <t xml:space="preserve">driver:otherPayGrowth</t>
         </is>
       </c>
       <c r="B242" s="2">
-        <v>0</v>
+        <v>0.02484645846924027</v>
       </c>
       <c r="C242" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:otherSgaRateEnd</t>
+          <t xml:space="preserve">driver:otherPayGrowthToBase</t>
         </is>
       </c>
       <c r="B243" s="2">
-        <v>0.005</v>
+        <v>0.01984645846924027</v>
       </c>
       <c r="C243" s="0" t="inlineStr">
         <is>
@@ -10470,26 +10512,26 @@
     <row r="244">
       <c r="A244" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectBaseYearSales</t>
+          <t xml:space="preserve">driver:otherResearchDevelopmentRate</t>
         </is>
       </c>
       <c r="B244" s="2">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="C244" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectCogsDepreciationShare</t>
+          <t xml:space="preserve">driver:otherSalesGrowth</t>
         </is>
       </c>
       <c r="B245" s="2">
-        <v>0.25</v>
+        <v>0.06257246376811586</v>
       </c>
       <c r="C245" s="0" t="inlineStr">
         <is>
@@ -10500,11 +10542,11 @@
     <row r="246">
       <c r="A246" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectCogsImprovementAfterBase</t>
+          <t xml:space="preserve">driver:otherSalesGrowthToBase</t>
         </is>
       </c>
       <c r="B246" s="2">
-        <v>0.015</v>
+        <v>0.042572463768115854</v>
       </c>
       <c r="C246" s="0" t="inlineStr">
         <is>
@@ -10515,26 +10557,26 @@
     <row r="247">
       <c r="A247" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectCogsImprovementToBase</t>
+          <t xml:space="preserve">driver:otherSgaImprovementToBase</t>
         </is>
       </c>
       <c r="B247" s="2">
-        <v>5.551115123125783e-17</v>
+        <v>0</v>
       </c>
       <c r="C247" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectCogsRateWhenSalesZero</t>
+          <t xml:space="preserve">driver:otherSgaRateEnd</t>
         </is>
       </c>
       <c r="B248" s="2">
-        <v>0.68</v>
+        <v>0.005</v>
       </c>
       <c r="C248" s="0" t="inlineStr">
         <is>
@@ -10545,56 +10587,56 @@
     <row r="249">
       <c r="A249" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectEmployeeSalaryShare</t>
+          <t xml:space="preserve">driver:projectBaseYearSales</t>
         </is>
       </c>
       <c r="B249" s="2">
-        <v>0.95</v>
+        <v>0</v>
       </c>
       <c r="C249" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectExtraordinaryRate</t>
+          <t xml:space="preserve">driver:projectCogsDepreciationShare</t>
         </is>
       </c>
       <c r="B250" s="2">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="C250" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectFirstYearSales</t>
+          <t xml:space="preserve">driver:projectCogsImprovementAfterBase</t>
         </is>
       </c>
       <c r="B251" s="2">
-        <v>0</v>
+        <v>0.015</v>
       </c>
       <c r="C251" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectHeadcountGrowth</t>
+          <t xml:space="preserve">driver:projectCogsImprovementToBase</t>
         </is>
       </c>
       <c r="B252" s="2">
-        <v>0.04</v>
+        <v>5.551115123125783e-17</v>
       </c>
       <c r="C252" s="0" t="inlineStr">
         <is>
@@ -10605,11 +10647,11 @@
     <row r="253">
       <c r="A253" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectHeadcountGrowthToBase</t>
+          <t xml:space="preserve">driver:projectCogsRateToBase</t>
         </is>
       </c>
       <c r="B253" s="2">
-        <v>0.05409356725146197</v>
+        <v>0.68</v>
       </c>
       <c r="C253" s="0" t="inlineStr">
         <is>
@@ -10620,11 +10662,11 @@
     <row r="254">
       <c r="A254" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectMarketGrowth</t>
+          <t xml:space="preserve">driver:projectCogsRateWhenSalesZero</t>
         </is>
       </c>
       <c r="B254" s="2">
-        <v>0.05</v>
+        <v>0.68</v>
       </c>
       <c r="C254" s="0" t="inlineStr">
         <is>
@@ -10635,56 +10677,56 @@
     <row r="255">
       <c r="A255" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectNonOperatingRate</t>
+          <t xml:space="preserve">driver:projectEmployeeSalaryShare</t>
         </is>
       </c>
       <c r="B255" s="2">
-        <v>0</v>
+        <v>0.95</v>
       </c>
       <c r="C255" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectOfficerCompensationShare</t>
+          <t xml:space="preserve">driver:projectExtraordinaryRate</t>
         </is>
       </c>
       <c r="B256" s="2">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="C256" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectOfficerPayGrowth</t>
+          <t xml:space="preserve">driver:projectFirstYearSales</t>
         </is>
       </c>
       <c r="B257" s="2">
-        <v>0.05380116959064325</v>
+        <v>0</v>
       </c>
       <c r="C257" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectOfficerPayGrowthToBase</t>
+          <t xml:space="preserve">driver:projectHeadcountGrowth</t>
         </is>
       </c>
       <c r="B258" s="2">
-        <v>0.05409356725146197</v>
+        <v>0.04</v>
       </c>
       <c r="C258" s="0" t="inlineStr">
         <is>
@@ -10695,11 +10737,11 @@
     <row r="259">
       <c r="A259" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectPayGrowth</t>
+          <t xml:space="preserve">driver:projectHeadcountGrowthToBase</t>
         </is>
       </c>
       <c r="B259" s="2">
-        <v>0.07</v>
+        <v>0.05409356725146197</v>
       </c>
       <c r="C259" s="0" t="inlineStr">
         <is>
@@ -10710,11 +10752,11 @@
     <row r="260">
       <c r="A260" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectPayGrowthToBase</t>
+          <t xml:space="preserve">driver:projectMarketGrowth</t>
         </is>
       </c>
       <c r="B260" s="2">
-        <v>0.020030662342518046</v>
+        <v>0.05</v>
       </c>
       <c r="C260" s="0" t="inlineStr">
         <is>
@@ -10725,26 +10767,26 @@
     <row r="261">
       <c r="A261" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectResearchDevelopmentRate</t>
+          <t xml:space="preserve">driver:projectNonOperatingRate</t>
         </is>
       </c>
       <c r="B261" s="2">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="C261" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectSalesGrowth</t>
+          <t xml:space="preserve">driver:projectOfficerCompensationShare</t>
         </is>
       </c>
       <c r="B262" s="2">
-        <v>0.22</v>
+        <v>0.9</v>
       </c>
       <c r="C262" s="0" t="inlineStr">
         <is>
@@ -10755,11 +10797,11 @@
     <row r="263">
       <c r="A263" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectSalesGrowthToBase</t>
+          <t xml:space="preserve">driver:projectOfficerPayGrowth</t>
         </is>
       </c>
       <c r="B263" s="2">
-        <v>0.05409356725146197</v>
+        <v>0.05380116959064325</v>
       </c>
       <c r="C263" s="0" t="inlineStr">
         <is>
@@ -10770,26 +10812,26 @@
     <row r="264">
       <c r="A264" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectSgaImprovementToBase</t>
+          <t xml:space="preserve">driver:projectOfficerPayGrowthToBase</t>
         </is>
       </c>
       <c r="B264" s="2">
-        <v>0</v>
+        <v>0.05409356725146197</v>
       </c>
       <c r="C264" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:projectSgaRateEnd</t>
+          <t xml:space="preserve">driver:projectPayGrowth</t>
         </is>
       </c>
       <c r="B265" s="2">
-        <v>0.015</v>
+        <v>0.07</v>
       </c>
       <c r="C265" s="0" t="inlineStr">
         <is>
@@ -10800,11 +10842,11 @@
     <row r="266">
       <c r="A266" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">driver:subsidy</t>
+          <t xml:space="preserve">driver:projectPayGrowthToBase</t>
         </is>
       </c>
       <c r="B266" s="2">
-        <v>766000</v>
+        <v>0.020030662342518046</v>
       </c>
       <c r="C266" s="0" t="inlineStr">
         <is>
@@ -10815,11 +10857,11 @@
     <row r="267">
       <c r="A267" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companyPaySchedule:max</t>
+          <t xml:space="preserve">driver:projectResearchDevelopmentRate</t>
         </is>
       </c>
       <c r="B267" s="2">
-        <v>7</v>
+        <v>0.005</v>
       </c>
       <c r="C267" s="0" t="inlineStr">
         <is>
@@ -10830,11 +10872,11 @@
     <row r="268">
       <c r="A268" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companyPaySchedule:value</t>
+          <t xml:space="preserve">driver:projectSalesGrowth</t>
         </is>
       </c>
       <c r="B268" s="2">
-        <v>3.5</v>
+        <v>0.22</v>
       </c>
       <c r="C268" s="0" t="inlineStr">
         <is>
@@ -10845,11 +10887,11 @@
     <row r="269">
       <c r="A269" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesCagr:max</t>
+          <t xml:space="preserve">driver:projectSalesGrowthToBase</t>
         </is>
       </c>
       <c r="B269" s="2">
-        <v>35</v>
+        <v>0.05409356725146197</v>
       </c>
       <c r="C269" s="0" t="inlineStr">
         <is>
@@ -10860,26 +10902,26 @@
     <row r="270">
       <c r="A270" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesCagr:value</t>
+          <t xml:space="preserve">driver:projectSgaImprovementToBase</t>
         </is>
       </c>
       <c r="B270" s="2">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="C270" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesIncrease:max</t>
+          <t xml:space="preserve">driver:projectSgaRateEnd</t>
         </is>
       </c>
       <c r="B271" s="2">
-        <v>25269000</v>
+        <v>0.015</v>
       </c>
       <c r="C271" s="0" t="inlineStr">
         <is>
@@ -10890,11 +10932,11 @@
     <row r="272">
       <c r="A272" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:companySalesIncrease:value</t>
+          <t xml:space="preserve">driver:subsidy</t>
         </is>
       </c>
       <c r="B272" s="2">
-        <v>8240000</v>
+        <v>766000</v>
       </c>
       <c r="C272" s="0" t="inlineStr">
         <is>
@@ -10905,11 +10947,11 @@
     <row r="273">
       <c r="A273" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayCagr:max</t>
+          <t xml:space="preserve">target:companyPaySchedule:max</t>
         </is>
       </c>
       <c r="B273" s="2">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C273" s="0" t="inlineStr">
         <is>
@@ -10920,11 +10962,11 @@
     <row r="274">
       <c r="A274" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayCagr:value</t>
+          <t xml:space="preserve">target:companyPaySchedule:value</t>
         </is>
       </c>
       <c r="B274" s="2">
-        <v>7</v>
+        <v>3.5</v>
       </c>
       <c r="C274" s="0" t="inlineStr">
         <is>
@@ -10935,11 +10977,11 @@
     <row r="275">
       <c r="A275" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayIncrease:max</t>
+          <t xml:space="preserve">target:companySalesCagr:max</t>
         </is>
       </c>
       <c r="B275" s="2">
-        <v>374000</v>
+        <v>35</v>
       </c>
       <c r="C275" s="0" t="inlineStr">
         <is>
@@ -10950,11 +10992,11 @@
     <row r="276">
       <c r="A276" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:employeePayIncrease:value</t>
+          <t xml:space="preserve">target:companySalesCagr:value</t>
         </is>
       </c>
       <c r="B276" s="2">
-        <v>285000</v>
+        <v>15</v>
       </c>
       <c r="C276" s="0" t="inlineStr">
         <is>
@@ -10965,11 +11007,11 @@
     <row r="277">
       <c r="A277" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:investmentSalesRatio:max</t>
+          <t xml:space="preserve">target:companySalesIncrease:max</t>
         </is>
       </c>
       <c r="B277" s="2">
-        <v>70</v>
+        <v>25269000</v>
       </c>
       <c r="C277" s="0" t="inlineStr">
         <is>
@@ -10980,11 +11022,11 @@
     <row r="278">
       <c r="A278" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:investmentSalesRatio:value</t>
+          <t xml:space="preserve">target:companySalesIncrease:value</t>
         </is>
       </c>
       <c r="B278" s="2">
-        <v>15</v>
+        <v>8240000</v>
       </c>
       <c r="C278" s="0" t="inlineStr">
         <is>
@@ -10995,11 +11037,11 @@
     <row r="279">
       <c r="A279" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:laborProductivityCagr:max</t>
+          <t xml:space="preserve">target:employeePayCagr:max</t>
         </is>
       </c>
       <c r="B279" s="2">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="C279" s="0" t="inlineStr">
         <is>
@@ -11010,11 +11052,11 @@
     <row r="280">
       <c r="A280" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:laborProductivityCagr:value</t>
+          <t xml:space="preserve">target:employeePayCagr:value</t>
         </is>
       </c>
       <c r="B280" s="2">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="C280" s="0" t="inlineStr">
         <is>
@@ -11025,11 +11067,11 @@
     <row r="281">
       <c r="A281" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:localBenchmark:max</t>
+          <t xml:space="preserve">target:employeePayIncrease:max</t>
         </is>
       </c>
       <c r="B281" s="2">
-        <v>40</v>
+        <v>374000</v>
       </c>
       <c r="C281" s="0" t="inlineStr">
         <is>
@@ -11040,11 +11082,11 @@
     <row r="282">
       <c r="A282" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:localBenchmark:value</t>
+          <t xml:space="preserve">target:employeePayIncrease:value</t>
         </is>
       </c>
       <c r="B282" s="2">
-        <v>23</v>
+        <v>285000</v>
       </c>
       <c r="C282" s="0" t="inlineStr">
         <is>
@@ -11055,11 +11097,11 @@
     <row r="283">
       <c r="A283" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:officerPayCagr:max</t>
+          <t xml:space="preserve">target:investmentSalesRatio:max</t>
         </is>
       </c>
       <c r="B283" s="2">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="C283" s="0" t="inlineStr">
         <is>
@@ -11070,11 +11112,11 @@
     <row r="284">
       <c r="A284" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:officerPayCagr:value</t>
+          <t xml:space="preserve">target:investmentSalesRatio:value</t>
         </is>
       </c>
       <c r="B284" s="2">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="C284" s="0" t="inlineStr">
         <is>
@@ -11085,26 +11127,26 @@
     <row r="285">
       <c r="A285" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:officerPayIncrease:value</t>
+          <t xml:space="preserve">target:laborProductivityCagr:max</t>
         </is>
       </c>
       <c r="B285" s="2">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="C285" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">明示的な0</t>
+          <t xml:space="preserve">入力済み</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesCagr:max</t>
+          <t xml:space="preserve">target:laborProductivityCagr:value</t>
         </is>
       </c>
       <c r="B286" s="2">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="C286" s="0" t="inlineStr">
         <is>
@@ -11115,11 +11157,11 @@
     <row r="287">
       <c r="A287" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesCagr:value</t>
+          <t xml:space="preserve">target:localBenchmark:max</t>
         </is>
       </c>
       <c r="B287" s="2">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="C287" s="0" t="inlineStr">
         <is>
@@ -11130,11 +11172,11 @@
     <row r="288">
       <c r="A288" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesIncrease:max</t>
+          <t xml:space="preserve">target:localBenchmark:value</t>
         </is>
       </c>
       <c r="B288" s="2">
-        <v>13684000</v>
+        <v>23</v>
       </c>
       <c r="C288" s="0" t="inlineStr">
         <is>
@@ -11145,11 +11187,11 @@
     <row r="289">
       <c r="A289" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesIncrease:value</t>
+          <t xml:space="preserve">target:officerPayCagr:max</t>
         </is>
       </c>
       <c r="B289" s="2">
-        <v>7480000</v>
+        <v>10</v>
       </c>
       <c r="C289" s="0" t="inlineStr">
         <is>
@@ -11160,11 +11202,11 @@
     <row r="290">
       <c r="A290" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesShare:max</t>
+          <t xml:space="preserve">target:officerPayCagr:value</t>
         </is>
       </c>
       <c r="B290" s="2">
-        <v>95</v>
+        <v>6</v>
       </c>
       <c r="C290" s="0" t="inlineStr">
         <is>
@@ -11175,26 +11217,26 @@
     <row r="291">
       <c r="A291" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:projectSalesShare:value</t>
+          <t xml:space="preserve">target:officerPayIncrease:value</t>
         </is>
       </c>
       <c r="B291" s="2">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="C291" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">入力済み</t>
+          <t xml:space="preserve">明示的な0</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:valueAddedIncrease:max</t>
+          <t xml:space="preserve">target:projectSalesCagr:max</t>
         </is>
       </c>
       <c r="B292" s="2">
-        <v>3343000</v>
+        <v>35</v>
       </c>
       <c r="C292" s="0" t="inlineStr">
         <is>
@@ -11205,11 +11247,11 @@
     <row r="293">
       <c r="A293" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:valueAddedIncrease:value</t>
+          <t xml:space="preserve">target:projectSalesCagr:value</t>
         </is>
       </c>
       <c r="B293" s="2">
-        <v>1878000</v>
+        <v>22</v>
       </c>
       <c r="C293" s="0" t="inlineStr">
         <is>
@@ -11220,11 +11262,11 @@
     <row r="294">
       <c r="A294" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">target:valueAddedSubsidyRatio:max</t>
+          <t xml:space="preserve">target:projectSalesIncrease:max</t>
         </is>
       </c>
       <c r="B294" s="2">
-        <v>350</v>
+        <v>13684000</v>
       </c>
       <c r="C294" s="0" t="inlineStr">
         <is>
@@ -11235,13 +11277,103 @@
     <row r="295">
       <c r="A295" s="0" t="inlineStr">
         <is>
+          <t xml:space="preserve">target:projectSalesIncrease:value</t>
+        </is>
+      </c>
+      <c r="B295" s="2">
+        <v>7480000</v>
+      </c>
+      <c r="C295" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesShare:max</t>
+        </is>
+      </c>
+      <c r="B296" s="2">
+        <v>95</v>
+      </c>
+      <c r="C296" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:projectSalesShare:value</t>
+        </is>
+      </c>
+      <c r="B297" s="2">
+        <v>60</v>
+      </c>
+      <c r="C297" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:valueAddedIncrease:max</t>
+        </is>
+      </c>
+      <c r="B298" s="2">
+        <v>3343000</v>
+      </c>
+      <c r="C298" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:valueAddedIncrease:value</t>
+        </is>
+      </c>
+      <c r="B299" s="2">
+        <v>1878000</v>
+      </c>
+      <c r="C299" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">target:valueAddedSubsidyRatio:max</t>
+        </is>
+      </c>
+      <c r="B300" s="2">
+        <v>350</v>
+      </c>
+      <c r="C300" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">入力済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="0" t="inlineStr">
+        <is>
           <t xml:space="preserve">target:valueAddedSubsidyRatio:value</t>
         </is>
       </c>
-      <c r="B295" s="2">
+      <c r="B301" s="2">
         <v>213</v>
       </c>
-      <c r="C295" s="0" t="inlineStr">
+      <c r="C301" s="0" t="inlineStr">
         <is>
           <t xml:space="preserve">入力済み</t>
         </is>
@@ -11269,14 +11401,14 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsIm1vbmV5VW5pdCI6IuWNg+WGhiIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOS4gOmDqOebruaomeacqumBlOOCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MjAwMDAwLCJjb2dzIjo0ODk2MDAwLCJlbXBsb3llZVBheSI6NTE5MDMxLCJvZmZpY2VyUGF5IjozNjAwMCwiZGVwcmVjaWF0aW9uIjoxODAwMDAsIm90aGVyU2dhIjo5MDAwMDAsImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQ5MzA3OSwiZW1wbG95ZWVCb251cyI6MjU5NTIsIm9mZmljZXJDb21wZW5zYXRpb24iOjMyNDAwLCJvZmZpY2VyQm9udXMiOjM2MDAsImNvZ3NEZXByZWNpYXRpb24iOjQ1MDAwLCJzZ2FEZXByZWNpYXRpb24iOjEzNTAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6MzYwMDB9LCJvdGhlciI6eyJzYWxlcyI6NjQ0MDAwMCwiY29ncyI6NDM3OTIwMCwiZW1wbG95ZWVQYXkiOjcwOTc4Niwib2ZmaWNlclBheSI6NTUyMDAsImRlcHJlY2lhdGlvbiI6MTM4MDAwLCJvdGhlclNnYSI6NzM2MDAwLCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Njc0Mjk3LCJlbXBsb3llZUJvbnVzIjozNTQ4OSwib2ZmaWNlckNvbXBlbnNhdGlvbiI6NDk2ODAsIm9mZmljZXJCb251cyI6NTUyMCwiY29nc0RlcHJlY2lhdGlvbiI6Mjc2MDAsInNnYURlcHJlY2lhdGlvbiI6MTEwNDAwLCJyZXNlYXJjaERldmVsb3BtZW50IjoyNzYwMCwib3JkaW5hcnlJbmNvbWUiOjM5NDUzNCwicHJlVGF4SW5jb21lIjozOTQ1MzQsIm5ldEluY29tZSI6NzUwNzUyLjF9fSx7InllYXIiOjIwMjQsInJvbGUiOiJwcmV2aW91cyIsInByb2plY3QiOnsic2FsZXMiOjc2MDAwMDAsImNvZ3MiOjUxNjgwMDAsImVtcGxveWVlUGF5Ijo1NTg4MjQsIm9mZmljZXJQYXkiOjM4MDAwLCJkZXByZWNpYXRpb24iOjE5MDAwMCwib3RoZXJTZ2EiOjk1MDAwMCwiaGVhZGNvdW50Ijo5NSwib2ZmaWNlckNvdW50IjoyLCJlbXBsb3llZVNhbGFyeSI6NTMwODgzLCJlbXBsb3llZUJvbnVzIjoyNzk0MSwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MzQyMDAsIm9mZmljZXJCb251cyI6MzgwMCwiY29nc0RlcHJlY2lhdGlvbiI6NDc1MDAsInNnYURlcHJlY2lhdGlvbiI6MTQyNTAwLCJyZXNlYXJjaERldmVsb3BtZW50IjozODAwMH0sIm90aGVyIjp7InNhbGVzIjo2NzIwMDAwLCJjb2dzIjo0NTY5NjAwLCJlbXBsb3llZVBheSI6NzU0MTQ4LCJvZmZpY2VyUGF5Ijo1NzYwMCwiZGVwcmVjaWF0aW9uIjoxNDQwMDAsIm90aGVyU2dhIjo3NjgwMDAsImhlYWRjb3VudCI6MTI1LCJvZmZpY2VyQ291bnQiOjMsImVtcGxveWVlU2FsYXJ5Ijo3MTY0NDEsImVtcGxveWVlQm9udXMiOjM3NzA3LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjo1MTg0MCwib2ZmaWNlckJvbnVzIjo1NzYwLCJjb2dzRGVwcmVjaWF0aW9uIjoyODgwMCwic2dhRGVwcmVjaWF0aW9uIjoxMTUyMDAsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjI4ODAwLCJvcmRpbmFyeUluY29tZSI6Mzk4MDEyLCJwcmVUYXhJbmNvbWUiOjM5ODAxMiwibmV0SW5jb21lIjo3NzE4ODEuNn19LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwMDAwMDAsImNvZ3MiOjU0NDAwMDAsImVtcGxveWVlUGF5Ijo2MDAwMDAsImVtcGxveWVlU2FsYXJ5Ijo1NzAwMDAsImVtcGxveWVlQm9udXMiOjMwMDAwLCJvZmZpY2VyUGF5Ijo0MDAwMCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MzYwMDAsIm9mZmljZXJCb251cyI6NDAwMCwiZGVwcmVjaWF0aW9uIjoyMDAwMDAsImNvZ3NEZXByZWNpYXRpb24iOjUwMDAwLCJzZ2FEZXByZWNpYXRpb24iOjE1MDAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6NDAwMDAsIm90aGVyU2dhIjoxMDAwMDAwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwMDAwMDAsImNvZ3MiOjQ3NjAwMDAsImVtcGxveWVlUGF5Ijo4MDAwMDAsImVtcGxveWVlU2FsYXJ5Ijo3NjAwMDAsImVtcGxveWVlQm9udXMiOjQwMDAwLCJvZmZpY2VyUGF5Ijo2MDAwMCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6NTQwMDAsIm9mZmljZXJCb251cyI6NjAwMCwiZGVwcmVjaWF0aW9uIjoxNTAwMDAsImNvZ3NEZXByZWNpYXRpb24iOjMwMDAwLCJzZ2FEZXByZWNpYXRpb24iOjEyMDAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6MzAwMDAsIm90aGVyU2dhIjo4MDAwMDAsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjo0MDAwMDAsInByZVRheEluY29tZSI6NDAwMDAwLCJuZXRJbmNvbWUiOjc5MTAwMH19XSwiYmFsYW5jZVNoZWV0cyI6W3sieWVhciI6MjAyMywiYXNzZXRzIjoxMzIwMDAwMCwiY3VycmVudEFzc2V0cyI6NjcwMDAwMCwiY2FzaCI6MjQwMDAwMCwiZml4ZWRBc3NldHMiOjY1MDAwMDAsInRhbmdpYmxlQXNzZXRzIjo1MzAwMDAwLCJidWlsZGluZ3MiOjE5MDAwMDAsIm1hY2hpbmVyeSI6MjQwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6NzAwMDAwLCJzb2Z0d2FyZSI6NTAwMDAwLCJsaWFiaWxpdGllcyI6NzUwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjozOTAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjozNjAwMDAwLCJsb25nVGVybURlYnQiOjI5MDAwMDAsIm5ldEFzc2V0cyI6NTcwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjU0MDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4Ijo1MDAwMDB9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMwMDAwMCwiY3VycmVudEFzc2V0cyI6NzIwMDAwMCwiY2FzaCI6MjUwMDAwMCwiZml4ZWRBc3NldHMiOjcxMDAwMDAsInRhbmdpYmxlQXNzZXRzIjo1ODAwMDAwLCJidWlsZGluZ3MiOjIwMDAwMDAsIm1hY2hpbmVyeSI6MjgwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6ODAwMDAwLCJzb2Z0d2FyZSI6NjAwMDAwLCJsaWFiaWxpdGllcyI6NzkwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjo0MTAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjozODAwMDAwLCJsb25nVGVybURlYnQiOjMxMDAwMDAsIm5ldEFzc2V0cyI6NjQwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjYxMDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4Ijo4MDAwMDB9LHsieWVhciI6MjAyNSwiYXNzZXRzIjoxNTYwMDAwMCwiY3VycmVudEFzc2V0cyI6NzgwMDAwMCwiY2FzaCI6MjcwMDAwMCwiZml4ZWRBc3NldHMiOjc4MDAwMDAsInRhbmdpYmxlQXNzZXRzIjo2NDAwMDAwLCJidWlsZGluZ3MiOjIyMDAwMDAsIm1hY2hpbmVyeSI6MzIwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6OTAwMDAwLCJzb2Z0d2FyZSI6NzAwMDAwLCJsaWFiaWxpdGllcyI6ODMwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjo0MzAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMTAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjo0MDAwMDAwLCJsb25nVGVybURlYnQiOjMyMDAwMDAsIm5ldEFzc2V0cyI6NzMwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjcwMDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4IjoxMDAwMDAwfV0sImZ1dHVyZUNhcGV4IjpbeyJ5ZWFyIjoyMDI2LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI4LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI5LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDMwLCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDMxLCJ2YWx1ZSI6MH1dLCJkcml2ZXJzIjp7InByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsInByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsIm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwib3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJwcm9qZWN0T2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjowLjksIm90aGVyT2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjowLjksInByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMjUsIm90aGVyQ29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjIsInByb2plY3RSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDUsIm90aGVyUmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA0LCJwcm9qZWN0Tm9uT3BlcmF0aW5nUmF0ZSI6MCwib3RoZXJOb25PcGVyYXRpbmdSYXRlIjotMC4wMDUsInByb2plY3RFeHRyYW9yZGluYXJ5UmF0ZSI6MCwib3RoZXJFeHRyYW9yZGluYXJ5UmF0ZSI6MCwiZWZmZWN0aXZlVGF4UmF0ZSI6MC4zLCJwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsInByb2plY3RGaXJzdFllYXJTYWxlcyI6MCwicHJvamVjdEJhc2VZZWFyU2FsZXMiOjAsInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjUuNTUxMTE1MTIzMTI1NzgzZS0xNywicHJvamVjdFBheUdyb3d0aFRvQmFzZSI6MC4wMjAwMzA2NjIzNDI1MTgwNDYsInByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNTcyNDYzNzY4MTE1ODU0LCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODQ2NDU4NDY5MjQwMjcsIm90aGVyT2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwODMzMzMzMzMzMzMzMzksIm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RTYWxlc0dyb3d0aCI6MC4yMiwib3RoZXJTYWxlc0dyb3d0aCI6MC4wNjI1NzI0NjM3NjgxMTU4NiwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTUsIm90aGVyQ29nc0ltcHJvdmVtZW50IjowLjAwNSwicHJvamVjdFBheUdyb3d0aCI6MC4wNywib3RoZXJQYXlHcm93dGgiOjAuMDI0ODQ2NDU4NDY5MjQwMjcsIm90aGVyT2ZmaWNlclBheUdyb3d0aCI6MC4wNDUsInByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsIm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTgzMzMzMzMzMzMzMzM4NiwicHJvamVjdFNnYVJhdGVFbmQiOjAuMDE1LCJvdGhlclNnYVJhdGVFbmQiOjAuMDA1LCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwiaW52ZXN0bWVudCI6MjMwMDAwMCwic3Vic2lkeSI6NzY2MDAwLCJsb2NhbEJlbmNobWFyayI6MjN9LCJkcml2ZXJSYW5nZXMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6Wy0wLjA1LDAuM10sInByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOlswLjY2LDAuN10sIm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjpbMC42NiwwLjddLCJwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6WzAsMV0sIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6WzAsMV0sInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOlswLDFdLCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6WzAsMV0sInByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOlswLDFdLCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6WzAsMV0sInByb2plY3RSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6WzAsMC4zXSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6WzAsMC4zXSwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOlstMC41LDAuNV0sIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6Wy0wLjUsMC41XSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjpbLTAuNSwwLjVdLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjpbLTAuNSwwLjVdLCJlZmZlY3RpdmVUYXhSYXRlIjpbMCwwLjZdLCJwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwicHJvamVjdEZpcnN0WWVhclNhbGVzIjpbMCwxMDAwMDAwMDAwMF0sInByb2plY3RCYXNlWWVhclNhbGVzIjpbMCwxMDAwMDAwMDAwMF0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDEuNjY1MzM0NTM2OTM3NzM0OGUtMTZdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkzMjUzMzA1MDE4NDY5MjcsMC4wMjA3MzU5OTQxODMxODkxNjZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlswLjA0MDc2MDg2OTU2NTIxNzE4NCwwLjA0NDM4NDA1Nzk3MTAxNDUyXSwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDAwMTM0NTc1NTY5MzU4MTk3MzddLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MTM5NDU3MDIzNzE3NDQzLDAuMDIwNTUzNDU5OTE0NzYzMDk1XSwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjAzOTE2NjY2NjY2NjY2NjY4LDAuMDQyNTAwMDAwMDAwMDAwMDldLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbMC4xNSwwLjNdLCJvdGhlclNhbGVzR3Jvd3RoIjpbMC4wNjA3NjA4Njk1NjUyMTcxOSwwLjA2NDM4NDA1Nzk3MTAxNDUzXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMC4wMDUsMC4wMDUxMzQ1NzU1NjkzNTgxOTc1XSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDUsMC4xXSwib3RoZXJQYXlHcm93dGgiOlswLjAyNDEzOTQ1NzAyMzcxNzQ0NCwwLjAyNTU1MzQ1OTkxNDc2MzA5Nl0sIm90aGVyT2ZmaWNlclBheUdyb3d0aCI6WzAsMC4wOF0sInByb2plY3RIZWFkY291bnRHcm93dGgiOlswLDAuMDhdLCJvdGhlckhlYWRjb3VudEdyb3d0aCI6WzAuMDQ0MTY2NjY2NjY2NjY2NjgsMC4wNDc1MDAwMDAwMDAwMDAwOV0sInByb2plY3RTZ2FSYXRlRW5kIjpbMCwwLjAzXSwib3RoZXJTZ2FSYXRlRW5kIjpbMCwwLjAxXSwicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOlswLjA0MjYzMTU3ODk0NzM2ODM2LDAuMDY1NTU1NTU1NTU1NTU1NThdLCJpbnZlc3RtZW50IjpbMTUwMDAwMCwyMDAwMDAwMF0sInN1YnNpZHkiOlsxMDAwMDAsNTAwMDAwMF0sImxvY2FsQmVuY2htYXJrIjpbMCwxMDBdfSwidGFyZ2V0cyI6eyJjb21wYW55U2FsZXNDYWdyIjp7InZhbHVlIjoxNSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo4MjQwMDAwLCJtYXgiOjI1MjY5MDAwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVBheVNjaGVkdWxlIjp7InZhbHVlIjozLjUsIm1heCI6NywicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc1NoYXJlIjp7InZhbHVlIjo2MCwibWF4Ijo5NSwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0NhZ3IiOnsidmFsdWUiOjIyLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjc0ODAwMDAsIm1heCI6MTM2ODQwMDAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsYWJvclByb2R1Y3Rpdml0eUNhZ3IiOnsidmFsdWUiOjIxLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZEluY3JlYXNlIjp7InZhbHVlIjoxODc4MDAwLCJtYXgiOjMzNDMwMDAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUNhZ3IiOnsidmFsdWUiOjcsIm1heCI6MTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUluY3JlYXNlIjp7InZhbHVlIjoyODUwMDAsIm1heCI6Mzc0MDAwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiaW52ZXN0bWVudFNhbGVzUmF0aW8iOnsidmFsdWUiOjE1LCJtYXgiOjcwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZFN1YnNpZHlSYXRpbyI6eyJ2YWx1ZSI6MjEzLCJtYXgiOjM1MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImxvY2FsQmVuY2htYXJrIjp7InZhbHVlIjoyMywibWF4Ijo0MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlDYWdyIjp7InZhbHVlIjo2LCJtYXgiOjEwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUluY3JlYXNlIjp7InZhbHVlIjowLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfX0sImZvcmVjYXN0T3ZlcnJpZGVzIjp7IjIwMjk6b3RoZXI6c2FsZXMiOjg1MTMwMDAsIjIwMjk6cHJvamVjdDo3LTgiOjc5MDAwMH0sImZ1dHVyZUlucHV0QmFzaXMiOiJvdGhlciIsImlucHV0VmFsdWVzIjp7ImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xIjoxMzY0MDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTMiOjkyNzUyMDAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi00Ijo3MjYwMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTciOjMyNjUwMTcsImFjdHVhbDpjb21wYW55OjIwMjM6Mi05Ijo4MjA4MCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEwIjo5MTIwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTIiOjExNjczNzYsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMyI6NjE0NDEsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNCI6MjQ1NDAwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTUiOjYzNjAwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTgiOjEwNzI1MDMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xOSI6MTA3MjUwMywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTIwIjo3NTA3NTIuMSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTI3IjoyMTAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yOCI6NSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEiOjcyMDAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny00IjoyMzA0MDAwLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNiI6Njc3OTY5LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOCI6NTE5MDMxLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOSI6MzYwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjM6UDItNCI6NDUwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjM6UDItMTQiOjEzNTAwMCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEzIjo5MCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMSI6MTQzMjAwMDAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0zIjo5NzM3NjAwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItNCI6NzYzMDAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi03IjozNDUxMDcyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItOSI6ODYwNDAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMCI6OTU2MCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEyIjoxMjQ3MzI0LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTMiOjY1NjQ4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTQiOjI1NzcwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE1Ijo2NjgwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE4IjoxMTAyNjg4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTkiOjExMDI2ODgsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0yMCI6NzcxODgxLjYsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0yNyI6MjIwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xIjo3NjAwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNCI6MjQzMjAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTYiOjcwNDY3NiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTgiOjU1ODgyNCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTkiOjM4MDAwLCJhY3R1YWw6cHJvamVjdDoyMDI0OlAyLTQiOjQ3NTAwLCJhY3R1YWw6cHJvamVjdDoyMDI0OlAyLTE0IjoxNDI1MDAsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xMyI6OTUsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xNCI6MiwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEiOjE1MDAwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMyI6MTAyMDAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi00Ijo4MDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTciOjM2NDAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi05Ijo5MDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEwIjoxMDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEyIjoxMzMwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTMiOjcwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTQiOjI3MDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE1Ijo3MDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE4IjoxMTMwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTkiOjExMzAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yMCI6NzkxMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMjciOjIzMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTI4Ijo1LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMSI6ODAwMDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTQiOjI1NjAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny02Ijo3MzAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny04Ijo2MDAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny05Ijo0MDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTpQMi00Ijo1MDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTpQMi0xNCI6MTUwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMTMiOjEwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTE0IjoyLCJiYWxhbmNlLXNoZWV0OjIwMjM6YXNzZXRzIjoxMzIwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmN1cnJlbnRBc3NldHMiOjY3MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXNoIjoyNDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6Zml4ZWRBc3NldHMiOjY1MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzp0YW5naWJsZUFzc2V0cyI6NTMwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmJ1aWxkaW5ncyI6MTkwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOm1hY2hpbmVyeSI6MjQwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmxhbmQiOjEwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzppbnRhbmdpYmxlQXNzZXRzIjo3MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpzb2Z0d2FyZSI6NTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6bGlhYmlsaXRpZXMiOjc1MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50TGlhYmlsaXRpZXMiOjM5MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6Zml4ZWRMaWFiaWxpdGllcyI6MzYwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmxvbmdUZXJtRGVidCI6MjkwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOm5ldEFzc2V0cyI6NTcwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOnNoYXJlaG9sZGVyRXF1aXR5Ijo1NDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FwaXRhbCI6MTAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGV4Ijo1MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDphc3NldHMiOjE0MzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y3VycmVudEFzc2V0cyI6NzIwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmNhc2giOjI1MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZEFzc2V0cyI6NzEwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OnRhbmdpYmxlQXNzZXRzIjo1ODAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6YnVpbGRpbmdzIjoyMDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6bWFjaGluZXJ5IjoyODAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGFuZCI6MTAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmludGFuZ2libGVBc3NldHMiOjgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OnNvZnR3YXJlIjo2MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpsaWFiaWxpdGllcyI6NzkwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRMaWFiaWxpdGllcyI6NDEwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OnNob3J0VGVybURlYnQiOjEyMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZExpYWJpbGl0aWVzIjozODAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6bG9uZ1Rlcm1EZWJ0IjozMTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6bmV0QXNzZXRzIjo2NDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hhcmVob2xkZXJFcXVpdHkiOjYxMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBpdGFsIjoxMDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwZXgiOjgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmFzc2V0cyI6MTU2MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50QXNzZXRzIjo3ODAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FzaCI6MjcwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkQXNzZXRzIjo3ODAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6dGFuZ2libGVBc3NldHMiOjY0MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpidWlsZGluZ3MiOjIyMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTptYWNoaW5lcnkiOjMyMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpsYW5kIjoxMDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6aW50YW5naWJsZUFzc2V0cyI6OTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6c29mdHdhcmUiOjcwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmxpYWJpbGl0aWVzIjo4MzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudExpYWJpbGl0aWVzIjo0MzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hvcnRUZXJtRGVidCI6MTEwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkTGlhYmlsaXRpZXMiOjQwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpsb25nVGVybURlYnQiOjMyMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpuZXRBc3NldHMiOjczMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaGFyZWhvbGRlckVxdWl0eSI6NzAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhcGl0YWwiOjEwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBleCI6MTAwMDAwMCwiZHJpdmVyOnByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0TWFya2V0R3Jvd3RoOjAiOi0wLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDoxIjowLjMsImRyaXZlcjpwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybzowIjowLjY2LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybzoxIjowLjcsImRyaXZlcjpvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvOjAiOjAuNjYsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybzoxIjowLjcsImRyaXZlcjpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwiZHJpdmVyLXJhbmdlOnByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZToxIjoxLCJkcml2ZXI6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJkcml2ZXItcmFuZ2U6b3RoZXJFbXBsb3llZVNhbGFyeVNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOm90aGVyT2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlIjowLjksImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMjUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0RlcHJlY2lhdGlvblNoYXJlOjEiOjEsImRyaXZlcjpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGU6MSI6MC4zLCJkcml2ZXI6b3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlOjEiOjAuMywiZHJpdmVyOnByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdE5vbk9wZXJhdGluZ1JhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOnByb2plY3ROb25PcGVyYXRpbmdSYXRlOjEiOjAuNSwiZHJpdmVyOm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJOb25PcGVyYXRpbmdSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpvdGhlck5vbk9wZXJhdGluZ1JhdGU6MSI6MC41LCJkcml2ZXI6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlOjAiOi0wLjUsImRyaXZlci1yYW5nZTpwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6b3RoZXJFeHRyYW9yZGluYXJ5UmF0ZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOm90aGVyRXh0cmFvcmRpbmFyeVJhdGU6MSI6MC41LCJkcml2ZXI6ZWZmZWN0aXZlVGF4UmF0ZSI6MC4zLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZTowIjowLCJkcml2ZXItcmFuZ2U6ZWZmZWN0aXZlVGF4UmF0ZToxIjowLjYsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RGaXJzdFllYXJTYWxlcyI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RGaXJzdFllYXJTYWxlczowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEZpcnN0WWVhclNhbGVzOjEiOjEwMDAwMDAwMDAwLCJkcml2ZXI6cHJvamVjdEJhc2VZZWFyU2FsZXMiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0QmFzZVllYXJTYWxlczowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEJhc2VZZWFyU2FsZXM6MSI6MTAwMDAwMDAwMDAsImRyaXZlcjpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjU1MTExNTEyMzEyNTc4M2UtMTcsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjEuNjY1MzM0NTM2OTM3NzM0OGUtMTYsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MCI6MC4wMTkzMjUzMzA1MDE4NDY5MjcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNzM1OTk0MTgzMTg5MTY2LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wNTExNjk1OTA2NDMyNzQ3NTQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDU3MDE3NTQzODU5NjQ5MTksImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlIjowLjA0MjU3MjQ2Mzc2ODExNTg1NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MCI6MC4wNDA3NjA4Njk1NjUyMTcxODQsImRyaXZlci1yYW5nZTpvdGhlclNhbGVzR3Jvd3RoVG9CYXNlOjEiOjAuMDQ0Mzg0MDU3OTcxMDE0NTIsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZToxIjowLjAwMDEzNDU3NTU2OTM1ODE5NzM3LCJkcml2ZXI6b3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDE5ODQ2NDU4NDY5MjQwMjcsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aFRvQmFzZTowIjowLjAxOTEzOTQ1NzAyMzcxNzQ0MywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjEiOjAuMDIwNTUzNDU5OTE0NzYzMDk1LCJkcml2ZXI6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDgzMzMzMzMzMzMzMzM5LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MCI6MC4wMzkxNjY2NjY2NjY2NjY2OCwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlOjEiOjAuMDQyNTAwMDAwMDAwMDAwMDksImRyaXZlcjpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZToxIjowLCJkcml2ZXI6cHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNhbGVzR3Jvd3RoOjAiOjAuMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MSI6MC4zLCJkcml2ZXI6b3RoZXJTYWxlc0dyb3d0aCI6MC4wNjI1NzI0NjM3NjgxMTU4NiwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGg6MCI6MC4wNjA3NjA4Njk1NjUyMTcxOSwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGg6MSI6MC4wNjQzODQwNTc5NzEwMTQ1MywiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRBZnRlckJhc2UiOjAuMDE1LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZToxIjowLjAzLCJkcml2ZXI6b3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnQ6MCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDoxIjowLjAwNTEzNDU3NTU2OTM1ODE5NzUsImRyaXZlcjpwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDowIjowLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aDoxIjowLjEsImRyaXZlcjpvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoOjAiOjAuMDI0MTM5NDU3MDIzNzE3NDQ0LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MSI6MC4wMjU1NTM0NTk5MTQ3NjMwOTYsImRyaXZlcjpvdGhlck9mZmljZXJQYXlHcm93dGgiOjAuMDQ1LCJkcml2ZXItcmFuZ2U6b3RoZXJPZmZpY2VyUGF5R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGg6MSI6MC4wOCwiZHJpdmVyOnByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDQsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoOjEiOjAuMDgsImRyaXZlcjpvdGhlckhlYWRjb3VudEdyb3d0aCI6MC4wNDU4MzMzMzMzMzMzMzMzODYsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDowIjowLjA0NDE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGg6MSI6MC4wNDc1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOnByb2plY3RTZ2FSYXRlRW5kIjowLjAxNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0U2dhUmF0ZUVuZDoxIjowLjAzLCJkcml2ZXI6b3RoZXJTZ2FSYXRlRW5kIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyU2dhUmF0ZUVuZDowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjEiOjAuMDEsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDExNjk1OTA2NDMyNSwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjAiOjAuMDQyNjMxNTc4OTQ3MzY4MzYsImRyaXZlci1yYW5nZTpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aDoxIjowLjA2NTU1NTU1NTU1NTU1NTU4LCJkcml2ZXI6aW52ZXN0bWVudCI6MjMwMDAwMCwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MCI6MTUwMDAwMCwiZHJpdmVyLXJhbmdlOmludmVzdG1lbnQ6MSI6MjAwMDAwMDAsImRyaXZlcjpzdWJzaWR5Ijo3NjYwMDAsImRyaXZlci1yYW5nZTpzdWJzaWR5OjAiOjEwMDAwMCwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MSI6NTAwMDAwMCwiZHJpdmVyOmxvY2FsQmVuY2htYXJrIjoyMywiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjAiOjAsImRyaXZlci1yYW5nZTpsb2NhbEJlbmNobWFyazoxIjoxMDAsInRhcmdldDpjb21wYW55U2FsZXNDYWdyOnZhbHVlIjoxNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6bWF4IjozNSwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOnZhbHVlIjo4MjQwMDAwLCJ0YXJnZXQ6Y29tcGFueVBheVNjaGVkdWxlOnZhbHVlIjozLjUsInRhcmdldDpjb21wYW55UGF5U2NoZWR1bGU6bWF4Ijo3LCJ0YXJnZXQ6cHJvamVjdFNhbGVzU2hhcmU6dmFsdWUiOjYwLCJ0YXJnZXQ6cHJvamVjdFNhbGVzU2hhcmU6bWF4Ijo5NSwidGFyZ2V0OnByb2plY3RTYWxlc0NhZ3I6dmFsdWUiOjIyLCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2FncjptYXgiOjM1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzSW5jcmVhc2U6dmFsdWUiOjc0ODAwMDAsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6dmFsdWUiOjIxLCJ0YXJnZXQ6bGFib3JQcm9kdWN0aXZpdHlDYWdyOm1heCI6MzUsInRhcmdldDp2YWx1ZUFkZGVkSW5jcmVhc2U6dmFsdWUiOjE4NzgwMDAsInRhcmdldDplbXBsb3llZVBheUNhZ3I6dmFsdWUiOjcsInRhcmdldDplbXBsb3llZVBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6dmFsdWUiOjI4NTAwMCwidGFyZ2V0OmludmVzdG1lbnRTYWxlc1JhdGlvOnZhbHVlIjoxNSwidGFyZ2V0OmludmVzdG1lbnRTYWxlc1JhdGlvOm1heCI6NzAsInRhcmdldDp2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvOnZhbHVlIjoyMTMsInRhcmdldDp2YWx1ZUFkZGVkU3Vic2lkeVJhdGlvOm1heCI6MzUwLCJ0YXJnZXQ6bG9jYWxCZW5jaG1hcms6dmFsdWUiOjIzLCJ0YXJnZXQ6bG9jYWxCZW5jaG1hcms6bWF4Ijo0MCwidGFyZ2V0Om9mZmljZXJQYXlDYWdyOnZhbHVlIjo2LCJ0YXJnZXQ6b2ZmaWNlclBheUNhZ3I6bWF4IjoxMCwidGFyZ2V0Om9mZmljZXJQYXlJbmNyZWFzZTp2YWx1ZSI6MCwidGFyZ2V0OmNvbXBhbnlTYWxlc0luY3JlYXNlOm1heCI6MjUyNjkwMDAsInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTptYXgiOjEzNjg0MDAwLCJ0YXJnZXQ6dmFsdWVBZGRlZEluY3JlYXNlOm1heCI6MzM0MzAwMCwidGFyZ2V0OmVtcGxveWVlUGF5SW5jcmVhc2U6bWF4IjozNzQwMDB9LCJtZXRyaWNHcm91cEJhc2VzIjp7ImNvbXBhbnlTYWxlcyI6InJhdGUiLCJwcm9qZWN0U2FsZXMiOiJyYXRlIiwibGFib3JQcm9kdWN0aXZpdHkiOiJyYXRlIiwiZW1wbG95ZWVQYXkiOiJyYXRlIn0sImFwcGxpY2F0aW9uQ2F0ZWdvcnkiOiJnZW5lcmFsIiwiYWRqdXN0ZWREcml2ZXJzIjp7InByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsInByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjc5OTk5OTk5OTk5OTk5OSwib3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjc5OTk5OTk5OTk5OTk5OSwicHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6MC45NSwicHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJwcm9qZWN0Q29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjI1LCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yLCJwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGUiOjAuMDA1LCJvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNCwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOjAsIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6LTAuMDA1LCJwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGUiOjAsIm90aGVyRXh0cmFvcmRpbmFyeVJhdGUiOjAsImVmZmVjdGl2ZVRheFJhdGUiOjAuMywicHJvamVjdFNhbGVzR3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJwcm9qZWN0Rmlyc3RZZWFyU2FsZXMiOjAsInByb2plY3RCYXNlWWVhclNhbGVzIjowLCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50VG9CYXNlIjo1LjE2Mjc2NTUwNTQ1ODU0N2UtMTcsInByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwNzM1OTk0MTgzMTg5MTY2LCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1MjIwNzU1OTcxNTYxNTUsInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDU0MDkzNTY3MjUxNDYxOTcsIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNTcyNDYzNzY4MTE1ODU0LCJvdGhlckNvZ3NJbXByb3ZlbWVudFRvQmFzZSI6MCwib3RoZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDIwNTUzNDU5OTE0NzYzMDk1LCJvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsIm90aGVySGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA0MDYyNTAwMDAwMDAwMDA1LCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIwMjA4ODc1MDkxMzA3NSwib3RoZXJTYWxlc0dyb3d0aCI6MC4wNjI1NzI0NjM3NjgxMTU4NiwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTUsIm90aGVyQ29nc0ltcHJvdmVtZW50IjowLjAwNSwicHJvamVjdFBheUdyb3d0aCI6MC4wODMwMzczNTU1NDk1ODM0NCwib3RoZXJQYXlHcm93dGgiOjAuMDI0ODQ2NDU4NDY5MjQwMjcsIm90aGVyT2ZmaWNlclBheUdyb3d0aCI6MC4wNDUsInByb2plY3RIZWFkY291bnRHcm93dGgiOjAuMDIwOTMxMDg1MTAyMTYyMjcsIm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTgzMzMzMzMzMzMzMzM4NiwicHJvamVjdFNnYVJhdGVFbmQiOjAuMDE1LCJvdGhlclNnYVJhdGVFbmQiOjAuMDA1LCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aCI6MC4wNTM4MDQ0MzM1OTE2NTkxMiwiaW52ZXN0bWVudCI6MjMwMDAwMCwi</t>
+          <t xml:space="preserve">eyJmb3JtYXQiOiJncm93dGgtaW52ZXN0bWVudC1wcm9wb3NhbC92MSIsIm1vbmV5VW5pdCI6IuWNg+WGhiIsInRpdGxlIjoi5oiQ6ZW35oqV6LOH6KiI55S7IOS4gOmDqOebruaomeacqumBlOOCteODs+ODl+ODqyIsImV4cG9ydGVkQXQiOiIyMDI2LTA3LTIyVDAwOjAwOjAwLjAwMFoiLCJ0aW1lbGluZSI6eyJsYXRlc3RZZWFyIjoyMDI1LCJiYXNlWWVhciI6MjAyOH0sImhpc3RvcmljYWxQbGFuIjpbeyJ5ZWFyIjoyMDIzLCJyb2xlIjoicHJlUHJldmlvdXMiLCJwcm9qZWN0Ijp7InNhbGVzIjo3MjAwMDAwLCJjb2dzIjo0ODk2MDAwLCJlbXBsb3llZVBheSI6NTE5MDMxLCJvZmZpY2VyUGF5IjozNjAwMCwiZGVwcmVjaWF0aW9uIjoxODAwMDAsIm90aGVyU2dhIjo5MDAwMDAsImhlYWRjb3VudCI6OTAsIm9mZmljZXJDb3VudCI6MiwiZW1wbG95ZWVTYWxhcnkiOjQ5MzA3OSwiZW1wbG95ZWVCb251cyI6MjU5NTIsIm9mZmljZXJDb21wZW5zYXRpb24iOjMyNDAwLCJvZmZpY2VyQm9udXMiOjM2MDAsImNvZ3NEZXByZWNpYXRpb24iOjQ1MDAwLCJzZ2FEZXByZWNpYXRpb24iOjEzNTAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6MzYwMDB9LCJvdGhlciI6eyJzYWxlcyI6NjQ0MDAwMCwiY29ncyI6NDM3OTIwMCwiZW1wbG95ZWVQYXkiOjcwOTc4Niwib2ZmaWNlclBheSI6NTUyMDAsImRlcHJlY2lhdGlvbiI6MTM4MDAwLCJvdGhlclNnYSI6NzM2MDAwLCJoZWFkY291bnQiOjEyMCwib2ZmaWNlckNvdW50IjozLCJlbXBsb3llZVNhbGFyeSI6Njc0Mjk3LCJlbXBsb3llZUJvbnVzIjozNTQ4OSwib2ZmaWNlckNvbXBlbnNhdGlvbiI6NDk2ODAsIm9mZmljZXJCb251cyI6NTUyMCwiY29nc0RlcHJlY2lhdGlvbiI6Mjc2MDAsInNnYURlcHJlY2lhdGlvbiI6MTEwNDAwLCJyZXNlYXJjaERldmVsb3BtZW50IjoyNzYwMCwib3JkaW5hcnlJbmNvbWUiOjM5NDUzNCwicHJlVGF4SW5jb21lIjozOTQ1MzQsIm5ldEluY29tZSI6NzUwNzUyLjF9fSx7InllYXIiOjIwMjQsInJvbGUiOiJwcmV2aW91cyIsInByb2plY3QiOnsic2FsZXMiOjc2MDAwMDAsImNvZ3MiOjUxNjgwMDAsImVtcGxveWVlUGF5Ijo1NTg4MjQsIm9mZmljZXJQYXkiOjM4MDAwLCJkZXByZWNpYXRpb24iOjE5MDAwMCwib3RoZXJTZ2EiOjk1MDAwMCwiaGVhZGNvdW50Ijo5NSwib2ZmaWNlckNvdW50IjoyLCJlbXBsb3llZVNhbGFyeSI6NTMwODgzLCJlbXBsb3llZUJvbnVzIjoyNzk0MSwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MzQyMDAsIm9mZmljZXJCb251cyI6MzgwMCwiY29nc0RlcHJlY2lhdGlvbiI6NDc1MDAsInNnYURlcHJlY2lhdGlvbiI6MTQyNTAwLCJyZXNlYXJjaERldmVsb3BtZW50IjozODAwMH0sIm90aGVyIjp7InNhbGVzIjo2NzIwMDAwLCJjb2dzIjo0NTY5NjAwLCJlbXBsb3llZVBheSI6NzU0MTQ4LCJvZmZpY2VyUGF5Ijo1NzYwMCwiZGVwcmVjaWF0aW9uIjoxNDQwMDAsIm90aGVyU2dhIjo3NjgwMDAsImhlYWRjb3VudCI6MTI1LCJvZmZpY2VyQ291bnQiOjMsImVtcGxveWVlU2FsYXJ5Ijo3MTY0NDEsImVtcGxveWVlQm9udXMiOjM3NzA3LCJvZmZpY2VyQ29tcGVuc2F0aW9uIjo1MTg0MCwib2ZmaWNlckJvbnVzIjo1NzYwLCJjb2dzRGVwcmVjaWF0aW9uIjoyODgwMCwic2dhRGVwcmVjaWF0aW9uIjoxMTUyMDAsInJlc2VhcmNoRGV2ZWxvcG1lbnQiOjI4ODAwLCJvcmRpbmFyeUluY29tZSI6Mzk4MDEyLCJwcmVUYXhJbmNvbWUiOjM5ODAxMiwibmV0SW5jb21lIjo3NzE4ODEuNn19LHsieWVhciI6MjAyNSwicm9sZSI6ImxhdGVzdCIsInByb2plY3QiOnsic2FsZXMiOjgwMDAwMDAsImNvZ3MiOjU0NDAwMDAsImVtcGxveWVlUGF5Ijo2MDAwMDAsImVtcGxveWVlU2FsYXJ5Ijo1NzAwMDAsImVtcGxveWVlQm9udXMiOjMwMDAwLCJvZmZpY2VyUGF5Ijo0MDAwMCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6MzYwMDAsIm9mZmljZXJCb251cyI6NDAwMCwiZGVwcmVjaWF0aW9uIjoyMDAwMDAsImNvZ3NEZXByZWNpYXRpb24iOjUwMDAwLCJzZ2FEZXByZWNpYXRpb24iOjE1MDAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6NDAwMDAsIm90aGVyU2dhIjoxMDAwMDAwLCJoZWFkY291bnQiOjEwMCwib2ZmaWNlckNvdW50IjoyfSwib3RoZXIiOnsic2FsZXMiOjcwMDAwMDAsImNvZ3MiOjQ3NjAwMDAsImVtcGxveWVlUGF5Ijo4MDAwMDAsImVtcGxveWVlU2FsYXJ5Ijo3NjAwMDAsImVtcGxveWVlQm9udXMiOjQwMDAwLCJvZmZpY2VyUGF5Ijo2MDAwMCwib2ZmaWNlckNvbXBlbnNhdGlvbiI6NTQwMDAsIm9mZmljZXJCb251cyI6NjAwMCwiZGVwcmVjaWF0aW9uIjoxNTAwMDAsImNvZ3NEZXByZWNpYXRpb24iOjMwMDAwLCJzZ2FEZXByZWNpYXRpb24iOjEyMDAwMCwicmVzZWFyY2hEZXZlbG9wbWVudCI6MzAwMDAsIm90aGVyU2dhIjo4MDAwMDAsImhlYWRjb3VudCI6MTMwLCJvZmZpY2VyQ291bnQiOjMsIm9yZGluYXJ5SW5jb21lIjo0MDAwMDAsInByZVRheEluY29tZSI6NDAwMDAwLCJuZXRJbmNvbWUiOjc5MTAwMH19XSwiYmFsYW5jZVNoZWV0cyI6W3sieWVhciI6MjAyMywiYXNzZXRzIjoxMzIwMDAwMCwiY3VycmVudEFzc2V0cyI6NjcwMDAwMCwiY2FzaCI6MjQwMDAwMCwiZml4ZWRBc3NldHMiOjY1MDAwMDAsInRhbmdpYmxlQXNzZXRzIjo1MzAwMDAwLCJidWlsZGluZ3MiOjE5MDAwMDAsIm1hY2hpbmVyeSI6MjQwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6NzAwMDAwLCJzb2Z0d2FyZSI6NTAwMDAwLCJsaWFiaWxpdGllcyI6NzUwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjozOTAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjozNjAwMDAwLCJsb25nVGVybURlYnQiOjI5MDAwMDAsIm5ldEFzc2V0cyI6NTcwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjU0MDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4Ijo1MDAwMDB9LHsieWVhciI6MjAyNCwiYXNzZXRzIjoxNDMwMDAwMCwiY3VycmVudEFzc2V0cyI6NzIwMDAwMCwiY2FzaCI6MjUwMDAwMCwiZml4ZWRBc3NldHMiOjcxMDAwMDAsInRhbmdpYmxlQXNzZXRzIjo1ODAwMDAwLCJidWlsZGluZ3MiOjIwMDAwMDAsIm1hY2hpbmVyeSI6MjgwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6ODAwMDAwLCJzb2Z0d2FyZSI6NjAwMDAwLCJsaWFiaWxpdGllcyI6NzkwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjo0MTAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjozODAwMDAwLCJsb25nVGVybURlYnQiOjMxMDAwMDAsIm5ldEFzc2V0cyI6NjQwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjYxMDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4Ijo4MDAwMDB9LHsieWVhciI6MjAyNSwiYXNzZXRzIjoxNTYwMDAwMCwiY3VycmVudEFzc2V0cyI6NzgwMDAwMCwiY2FzaCI6MjcwMDAwMCwiZml4ZWRBc3NldHMiOjc4MDAwMDAsInRhbmdpYmxlQXNzZXRzIjo2NDAwMDAwLCJidWlsZGluZ3MiOjIyMDAwMDAsIm1hY2hpbmVyeSI6MzIwMDAwMCwibGFuZCI6MTAwMDAwMCwiaW50YW5naWJsZUFzc2V0cyI6OTAwMDAwLCJzb2Z0d2FyZSI6NzAwMDAwLCJsaWFiaWxpdGllcyI6ODMwMDAwMCwiY3VycmVudExpYWJpbGl0aWVzIjo0MzAwMDAwLCJzaG9ydFRlcm1EZWJ0IjoxMTAwMDAwLCJmaXhlZExpYWJpbGl0aWVzIjo0MDAwMDAwLCJsb25nVGVybURlYnQiOjMyMDAwMDAsIm5ldEFzc2V0cyI6NzMwMDAwMCwic2hhcmVob2xkZXJFcXVpdHkiOjcwMDAwMDAsImNhcGl0YWwiOjEwMDAwMDAsImNhcGV4IjoxMDAwMDAwfV0sImZ1dHVyZUNhcGV4IjpbeyJ5ZWFyIjoyMDI2LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI3LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI4LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDI5LCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDMwLCJ2YWx1ZSI6MH0seyJ5ZWFyIjoyMDMxLCJ2YWx1ZSI6MH1dLCJkcml2ZXJzIjp7InByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsInByb2plY3RDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOjAuNjgsIm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJwcm9qZWN0Q29nc1JhdGVUb0Jhc2UiOjAuNjgsIm90aGVyQ29nc1JhdGVUb0Jhc2UiOjAuNjgsInByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwib3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwicHJvamVjdENvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yNSwib3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMiwicHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsInByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJvdGhlck5vbk9wZXJhdGluZ1JhdGUiOi0wLjAwNSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjowLCJlZmZlY3RpdmVUYXhSYXRlIjowLjMsInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywicHJvamVjdEZpcnN0WWVhclNhbGVzIjowLCJwcm9qZWN0QmFzZVllYXJTYWxlcyI6MCwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6NS41NTExMTUxMjMxMjU3ODNlLTE3LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDAzMDY2MjM0MjUxODA0NiwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5Nywib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI1NzI0NjM3NjgxMTU4NTQsIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4NDY0NTg0NjkyNDAyNywib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjowLjA0LCJvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNDA4MzMzMzMzMzMzMzMzOSwib3RoZXJTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwicHJvamVjdFNhbGVzR3Jvd3RoIjowLjIyLCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA3LCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywib3RoZXJPZmZpY2VyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODMzMzMzMzMzMzMzMzg2LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4wMTUsIm90aGVyU2dhUmF0ZUVuZCI6MC4wMDUsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJpbnZlc3RtZW50IjoyMzAwMDAwLCJzdWJzaWR5Ijo3NjYwMDAsImxvY2FsQmVuY2htYXJrIjoyM30sImRyaXZlclJhbmdlcyI6eyJwcm9qZWN0TWFya2V0R3Jvd3RoIjpbLTAuMDUsMC4zXSwicHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6WzAuNjYsMC43XSwib3RoZXJDb2dzUmF0ZVdoZW5TYWxlc1plcm8iOlswLjY2LDAuN10sInByb2plY3RDb2dzUmF0ZVRvQmFzZSI6WzAuNjgsMC42OF0sIm90aGVyQ29nc1JhdGVUb0Jhc2UiOlswLjY4LDAuNjhdLCJwcm9qZWN0RW1wbG95ZWVTYWxhcnlTaGFyZSI6WzAsMV0sIm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZSI6WzAsMV0sInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOlswLDFdLCJvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6WzAsMV0sInByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOlswLDFdLCJvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZSI6WzAsMV0sInByb2plY3RSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6WzAsMC4zXSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6WzAsMC4zXSwicHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOlstMC41LDAuNV0sIm90aGVyTm9uT3BlcmF0aW5nUmF0ZSI6Wy0wLjUsMC41XSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjpbLTAuNSwwLjVdLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjpbLTAuNSwwLjVdLCJlZmZlY3RpdmVUYXhSYXRlIjpbMCwwLjZdLCJwcm9qZWN0U2FsZXNHcm93dGhUb0Jhc2UiOlswLjA1MTE2OTU5MDY0MzI3NDc1NCwwLjA1NzAxNzU0Mzg1OTY0OTE5XSwicHJvamVjdEZpcnN0WWVhclNhbGVzIjpbMCwxMDAwMDAwMDAwMF0sInByb2plY3RCYXNlWWVhclNhbGVzIjpbMCwxMDAwMDAwMDAwMF0sInByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDEuNjY1MzM0NTM2OTM3NzM0OGUtMTZdLCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjpbMC4wMTkzMjUzMzA1MDE4NDY5MjcsMC4wMjA3MzU5OTQxODMxODkxNjZdLCJwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sInByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6WzAsMF0sInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMC4wNTExNjk1OTA2NDMyNzQ3NTQsMC4wNTcwMTc1NDM4NTk2NDkxOV0sIm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOlswLjA0MDc2MDg2OTU2NTIxNzE4NCwwLjA0NDM4NDA1Nzk3MTAxNDUyXSwib3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOlswLDAuMDAwMTM0NTc1NTY5MzU4MTk3MzddLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6WzAuMDE5MTM5NDU3MDIzNzE3NDQzLDAuMDIwNTUzNDU5OTE0NzYzMDk1XSwib3RoZXJPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlIjpbMCwwLjA4XSwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOlswLjAzOTE2NjY2NjY2NjY2NjY4LDAuMDQyNTAwMDAwMDAwMDAwMDldLCJvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlIjpbMCwwXSwicHJvamVjdFNhbGVzR3Jvd3RoIjpbMC4xNSwwLjNdLCJvdGhlclNhbGVzR3Jvd3RoIjpbMC4wNjA3NjA4Njk1NjUyMTcxOSwwLjA2NDM4NDA1Nzk3MTAxNDUzXSwicHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6WzAsMC4wM10sIm90aGVyQ29nc0ltcHJvdmVtZW50IjpbMC4wMDUsMC4wMDUxMzQ1NzU1NjkzNTgxOTc1XSwicHJvamVjdFBheUdyb3d0aCI6WzAuMDUsMC4xXSwib3RoZXJQYXlHcm93dGgiOlswLjAyNDEzOTQ1NzAyMzcxNzQ0NCwwLjAyNTU1MzQ1OTkxNDc2MzA5Nl0sIm90aGVyT2ZmaWNlclBheUdyb3d0aCI6WzAsMC4wOF0sInByb2plY3RIZWFkY291bnRHcm93dGgiOlswLDAuMDhdLCJvdGhlckhlYWRjb3VudEdyb3d0aCI6WzAuMDQ0MTY2NjY2NjY2NjY2NjgsMC4wNDc1MDAwMDAwMDAwMDAwOV0sInByb2plY3RTZ2FSYXRlRW5kIjpbMCwwLjAzXSwib3RoZXJTZ2FSYXRlRW5kIjpbMCwwLjAxXSwicHJvamVjdE9mZmljZXJQYXlHcm93dGgiOlswLjA0MjYzMTU3ODk0NzM2ODM2LDAuMDY1NTU1NTU1NTU1NTU1NThdLCJpbnZlc3RtZW50IjpbMTUwMDAwMCwyMDAwMDAwMF0sInN1YnNpZHkiOlsxMDAwMDAsNTAwMDAwMF0sImxvY2FsQmVuY2htYXJrIjpbMCwxMDBdfSwidGFyZ2V0cyI6eyJjb21wYW55U2FsZXNDYWdyIjp7InZhbHVlIjoxNSwibWF4IjozNSwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImNvbXBhbnlTYWxlc0luY3JlYXNlIjp7InZhbHVlIjo4MjQwMDAwLCJtYXgiOjI1MjY5MDAwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiY29tcGFueVBheVNjaGVkdWxlIjp7InZhbHVlIjozLjUsIm1heCI6NywicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc1NoYXJlIjp7InZhbHVlIjo2MCwibWF4Ijo5NSwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sInByb2plY3RTYWxlc0NhZ3IiOnsidmFsdWUiOjIyLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwicHJvamVjdFNhbGVzSW5jcmVhc2UiOnsidmFsdWUiOjc0ODAwMDAsIm1heCI6MTM2ODQwMDAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJsYWJvclByb2R1Y3Rpdml0eUNhZ3IiOnsidmFsdWUiOjIxLCJtYXgiOjM1LCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZEluY3JlYXNlIjp7InZhbHVlIjoxODc4MDAwLCJtYXgiOjMzNDMwMDAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUNhZ3IiOnsidmFsdWUiOjcsIm1heCI6MTAsInBvbGljeSI6InNvZnQiLCJ3ZWlnaHQiOjF9LCJlbXBsb3llZVBheUluY3JlYXNlIjp7InZhbHVlIjoyODUwMDAsIm1heCI6Mzc0MDAwLCJwb2xpY3kiOiJzb2Z0Iiwid2VpZ2h0IjoxfSwiaW52ZXN0bWVudFNhbGVzUmF0aW8iOnsidmFsdWUiOjE1LCJtYXgiOjcwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwidmFsdWVBZGRlZFN1YnNpZHlSYXRpbyI6eyJ2YWx1ZSI6MjEzLCJtYXgiOjM1MCwicG9saWN5Ijoic29mdCIsIndlaWdodCI6MX0sImxvY2FsQmVuY2htYXJrIjp7InZhbHVlIjoyMywibWF4Ijo0MCwicG9saWN5IjoibW9uaXRvciIsIndlaWdodCI6MX0sIm9mZmljZXJQYXlDYWdyIjp7InZhbHVlIjo2LCJtYXgiOjEwLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfSwib2ZmaWNlclBheUluY3JlYXNlIjp7InZhbHVlIjowLCJwb2xpY3kiOiJtb25pdG9yIiwid2VpZ2h0IjoxfX0sImZvcmVjYXN0T3ZlcnJpZGVzIjp7IjIwMjk6b3RoZXI6c2FsZXMiOjg1MTMwMDAsIjIwMjk6cHJvamVjdDo3LTgiOjc5MDAwMH0sImZ1dHVyZUlucHV0QmFzaXMiOiJvdGhlciIsImlucHV0VmFsdWVzIjp7ImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xIjoxMzY0MDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTMiOjkyNzUyMDAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi00Ijo3MjYwMCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTciOjMyNjUwMTcsImFjdHVhbDpjb21wYW55OjIwMjM6Mi05Ijo4MjA4MCwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTEwIjo5MTIwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTIiOjExNjczNzYsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xMyI6NjE0NDEsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xNCI6MjQ1NDAwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTUiOjYzNjAwLCJhY3R1YWw6Y29tcGFueToyMDIzOjItMTgiOjEwNzI1MDMsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0xOSI6MTA3MjUwMywiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTIwIjo3NTA3NTIuMSwiYWN0dWFsOmNvbXBhbnk6MjAyMzoyLTI3IjoyMTAsImFjdHVhbDpjb21wYW55OjIwMjM6Mi0yOCI6NSwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEiOjcyMDAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjM6Ny00IjoyMzA0MDAwLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctNiI6Njc3OTY5LCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOCI6NTE5MDMxLCJhY3R1YWw6cHJvamVjdDoyMDIzOjctOSI6MzYwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjM6UDItNCI6NDUwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjM6UDItMTQiOjEzNTAwMCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTEzIjo5MCwiYWN0dWFsOnByb2plY3Q6MjAyMzo3LTE0IjoyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMSI6MTQzMjAwMDAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0zIjo5NzM3NjAwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItNCI6NzYzMDAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi03IjozNDUxMDcyLCJhY3R1YWw6Y29tcGFueToyMDI0OjItOSI6ODYwNDAsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0xMCI6OTU2MCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTEyIjoxMjQ3MzI0LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTMiOjY1NjQ4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTQiOjI1NzcwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE1Ijo2NjgwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNDoyLTE4IjoxMTAyNjg4LCJhY3R1YWw6Y29tcGFueToyMDI0OjItMTkiOjExMDI2ODgsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0yMCI6NzcxODgxLjYsImFjdHVhbDpjb21wYW55OjIwMjQ6Mi0yNyI6MjIwLCJhY3R1YWw6Y29tcGFueToyMDI0OjItMjgiOjUsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xIjo3NjAwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDI0OjctNCI6MjQzMjAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTYiOjcwNDY3NiwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTgiOjU1ODgyNCwiYWN0dWFsOnByb2plY3Q6MjAyNDo3LTkiOjM4MDAwLCJhY3R1YWw6cHJvamVjdDoyMDI0OlAyLTQiOjQ3NTAwLCJhY3R1YWw6cHJvamVjdDoyMDI0OlAyLTE0IjoxNDI1MDAsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xMyI6OTUsImFjdHVhbDpwcm9qZWN0OjIwMjQ6Ny0xNCI6MiwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEiOjE1MDAwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMyI6MTAyMDAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi00Ijo4MDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTciOjM2NDAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi05Ijo5MDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEwIjoxMDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTEyIjoxMzMwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTMiOjcwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTQiOjI3MDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE1Ijo3MDAwMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTE4IjoxMTMwMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMTkiOjExMzAwMDAsImFjdHVhbDpjb21wYW55OjIwMjU6Mi0yMCI6NzkxMDAwLCJhY3R1YWw6Y29tcGFueToyMDI1OjItMjciOjIzMCwiYWN0dWFsOmNvbXBhbnk6MjAyNToyLTI4Ijo1LCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMSI6ODAwMDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTQiOjI1NjAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny02Ijo3MzAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny04Ijo2MDAwMDAsImFjdHVhbDpwcm9qZWN0OjIwMjU6Ny05Ijo0MDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTpQMi00Ijo1MDAwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTpQMi0xNCI6MTUwMDAwLCJhY3R1YWw6cHJvamVjdDoyMDI1OjctMTMiOjEwMCwiYWN0dWFsOnByb2plY3Q6MjAyNTo3LTE0IjoyLCJiYWxhbmNlLXNoZWV0OjIwMjM6YXNzZXRzIjoxMzIwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmN1cnJlbnRBc3NldHMiOjY3MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjYXNoIjoyNDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6Zml4ZWRBc3NldHMiOjY1MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzp0YW5naWJsZUFzc2V0cyI6NTMwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmJ1aWxkaW5ncyI6MTkwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOm1hY2hpbmVyeSI6MjQwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmxhbmQiOjEwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzppbnRhbmdpYmxlQXNzZXRzIjo3MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpzb2Z0d2FyZSI6NTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6bGlhYmlsaXRpZXMiOjc1MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpjdXJyZW50TGlhYmlsaXRpZXMiOjM5MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyMzpzaG9ydFRlcm1EZWJ0IjoxMjAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6Zml4ZWRMaWFiaWxpdGllcyI6MzYwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmxvbmdUZXJtRGVidCI6MjkwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOm5ldEFzc2V0cyI6NTcwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOnNoYXJlaG9sZGVyRXF1aXR5Ijo1NDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjM6Y2FwaXRhbCI6MTAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDIzOmNhcGV4Ijo1MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDphc3NldHMiOjE0MzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y3VycmVudEFzc2V0cyI6NzIwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmNhc2giOjI1MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZEFzc2V0cyI6NzEwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OnRhbmdpYmxlQXNzZXRzIjo1ODAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6YnVpbGRpbmdzIjoyMDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6bWFjaGluZXJ5IjoyODAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6bGFuZCI6MTAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmludGFuZ2libGVBc3NldHMiOjgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OnNvZnR3YXJlIjo2MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpsaWFiaWxpdGllcyI6NzkwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OmN1cnJlbnRMaWFiaWxpdGllcyI6NDEwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI0OnNob3J0VGVybURlYnQiOjEyMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpmaXhlZExpYWJpbGl0aWVzIjozODAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6bG9uZ1Rlcm1EZWJ0IjozMTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6bmV0QXNzZXRzIjo2NDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6c2hhcmVob2xkZXJFcXVpdHkiOjYxMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNDpjYXBpdGFsIjoxMDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjQ6Y2FwZXgiOjgwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmFzc2V0cyI6MTU2MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjdXJyZW50QXNzZXRzIjo3ODAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y2FzaCI6MjcwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkQXNzZXRzIjo3ODAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6dGFuZ2libGVBc3NldHMiOjY0MDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpidWlsZGluZ3MiOjIyMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTptYWNoaW5lcnkiOjMyMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpsYW5kIjoxMDAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6aW50YW5naWJsZUFzc2V0cyI6OTAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6c29mdHdhcmUiOjcwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmxpYWJpbGl0aWVzIjo4MzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6Y3VycmVudExpYWJpbGl0aWVzIjo0MzAwMDAwLCJiYWxhbmNlLXNoZWV0OjIwMjU6c2hvcnRUZXJtRGVidCI6MTEwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmZpeGVkTGlhYmlsaXRpZXMiOjQwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpsb25nVGVybURlYnQiOjMyMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpuZXRBc3NldHMiOjczMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpzaGFyZWhvbGRlckVxdWl0eSI6NzAwMDAwMCwiYmFsYW5jZS1zaGVldDoyMDI1OmNhcGl0YWwiOjEwMDAwMDAsImJhbGFuY2Utc2hlZXQ6MjAyNTpjYXBleCI6MTAwMDAwMCwiZHJpdmVyOnByb2plY3RNYXJrZXRHcm93dGgiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0TWFya2V0R3Jvd3RoOjAiOi0wLjA1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE1hcmtldEdyb3d0aDoxIjowLjMsImRyaXZlcjpwcm9qZWN0Q29nc1JhdGVXaGVuU2FsZXNaZXJvIjowLjY4LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybzowIjowLjY2LCJkcml2ZXItcmFuZ2U6cHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybzoxIjowLjcsImRyaXZlcjpvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42OCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc1JhdGVXaGVuU2FsZXNaZXJvOjAiOjAuNjYsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybzoxIjowLjcsImRyaXZlcjpwcm9qZWN0Q29nc1JhdGVUb0Jhc2UiOjAuNjgsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc1JhdGVUb0Jhc2U6MCI6MC42OCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzUmF0ZVRvQmFzZToxIjowLjY4LCJkcml2ZXI6b3RoZXJDb2dzUmF0ZVRvQmFzZSI6MC42OCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc1JhdGVUb0Jhc2U6MCI6MC42OCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc1JhdGVUb0Jhc2U6MSI6MC42OCwiZHJpdmVyOnByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJkcml2ZXItcmFuZ2U6cHJvamVjdEVtcGxveWVlU2FsYXJ5U2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlOjEiOjEsImRyaXZlcjpvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsImRyaXZlci1yYW5nZTpvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyRW1wbG95ZWVTYWxhcnlTaGFyZToxIjoxLCJkcml2ZXI6cHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZSI6MC45LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJDb21wZW5zYXRpb25TaGFyZToxIjoxLCJkcml2ZXI6b3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlckNvbXBlbnNhdGlvblNoYXJlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJDb21wZW5zYXRpb25TaGFyZToxIjoxLCJkcml2ZXI6cHJvamVjdENvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yNSwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmU6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzRGVwcmVjaWF0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOm90aGVyQ29nc0RlcHJlY2lhdGlvblNoYXJlIjowLjIsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NEZXByZWNpYXRpb25TaGFyZTowIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmU6MSI6MSwiZHJpdmVyOnByb2plY3RSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0UmVzZWFyY2hEZXZlbG9wbWVudFJhdGU6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RSZXNlYXJjaERldmVsb3BtZW50UmF0ZToxIjowLjMsImRyaXZlcjpvdGhlclJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNCwiZHJpdmVyLXJhbmdlOm90aGVyUmVzZWFyY2hEZXZlbG9wbWVudFJhdGU6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyUmVzZWFyY2hEZXZlbG9wbWVudFJhdGU6MSI6MC4zLCJkcml2ZXI6cHJvamVjdE5vbk9wZXJhdGluZ1JhdGUiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Tm9uT3BlcmF0aW5nUmF0ZTowIjotMC41LCJkcml2ZXItcmFuZ2U6cHJvamVjdE5vbk9wZXJhdGluZ1JhdGU6MSI6MC41LCJkcml2ZXI6b3RoZXJOb25PcGVyYXRpbmdSYXRlIjotMC4wMDUsImRyaXZlci1yYW5nZTpvdGhlck5vbk9wZXJhdGluZ1JhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOm90aGVyTm9uT3BlcmF0aW5nUmF0ZToxIjowLjUsImRyaXZlcjpwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGUiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0RXh0cmFvcmRpbmFyeVJhdGU6MCI6LTAuNSwiZHJpdmVyLXJhbmdlOnByb2plY3RFeHRyYW9yZGluYXJ5UmF0ZToxIjowLjUsImRyaXZlcjpvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJFeHRyYW9yZGluYXJ5UmF0ZTowIjotMC41LCJkcml2ZXItcmFuZ2U6b3RoZXJFeHRyYW9yZGluYXJ5UmF0ZToxIjowLjUsImRyaXZlcjplZmZlY3RpdmVUYXhSYXRlIjowLjMsImRyaXZlci1yYW5nZTplZmZlY3RpdmVUYXhSYXRlOjAiOjAsImRyaXZlci1yYW5nZTplZmZlY3RpdmVUYXhSYXRlOjEiOjAuNiwiZHJpdmVyOnByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aFRvQmFzZToxIjowLjA1NzAxNzU0Mzg1OTY0OTE5LCJkcml2ZXI6cHJvamVjdEZpcnN0WWVhclNhbGVzIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdEZpcnN0WWVhclNhbGVzOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Rmlyc3RZZWFyU2FsZXM6MSI6MTAwMDAwMDAwMDAsImRyaXZlcjpwcm9qZWN0QmFzZVllYXJTYWxlcyI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RCYXNlWWVhclNhbGVzOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0QmFzZVllYXJTYWxlczoxIjoxMDAwMDAwMDAwMCwiZHJpdmVyOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2UiOjUuNTUxMTE1MTIzMTI1NzgzZS0xNywiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MSI6MS42NjUzMzQ1MzY5Mzc3MzQ4ZS0xNiwiZHJpdmVyOnByb2plY3RQYXlHcm93dGhUb0Jhc2UiOjAuMDIwMDMwNjYyMzQyNTE4MDQ2LCJkcml2ZXItcmFuZ2U6cHJvamVjdFBheUdyb3d0aFRvQmFzZTowIjowLjAxOTMyNTMzMDUwMTg0NjkyNywiZHJpdmVyLXJhbmdlOnByb2plY3RQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA3MzU5OTQxODMxODkxNjYsImRyaXZlcjpwcm9qZWN0SGVhZGNvdW50R3Jvd3RoVG9CYXNlIjowLjA1NDA5MzU2NzI1MTQ2MTk3LCJkcml2ZXItcmFuZ2U6cHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjA1MTE2OTU5MDY0MzI3NDc1NCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZSI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FJbXByb3ZlbWVudFRvQmFzZTowIjowLCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDUxMTY5NTkwNjQzMjc0NzU0LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wNTcwMTc1NDM4NTk2NDkxOSwiZHJpdmVyOm90aGVyU2FsZXNHcm93dGhUb0Jhc2UiOjAuMDQyNTcyNDYzNzY4MTE1ODU0LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aFRvQmFzZTowIjowLjA0MDc2MDg2OTU2NTIxNzE4NCwiZHJpdmVyLXJhbmdlOm90aGVyU2FsZXNHcm93dGhUb0Jhc2U6MSI6MC4wNDQzODQwNTc5NzEwMTQ1MiwiZHJpdmVyOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJkcml2ZXItcmFuZ2U6b3RoZXJDb2dzSW1wcm92ZW1lbnRUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlOjEiOjAuMDAwMTM0NTc1NTY5MzU4MTk3MzcsImRyaXZlcjpvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMTk4NDY0NTg0NjkyNDAyNywiZHJpdmVyLXJhbmdlOm90aGVyUGF5R3Jvd3RoVG9CYXNlOjAiOjAuMDE5MTM5NDU3MDIzNzE3NDQzLCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGhUb0Jhc2U6MSI6MC4wMjA1NTM0NTk5MTQ3NjMwOTUsImRyaXZlcjpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2UiOjAuMDQsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGhUb0Jhc2U6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlclBheUdyb3d0aFRvQmFzZToxIjowLjA4LCJkcml2ZXI6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwODMzMzMzMzMzMzMzMzksImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aFRvQmFzZTowIjowLjAzOTE2NjY2NjY2NjY2NjY4LCJkcml2ZXItcmFuZ2U6b3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2U6MSI6MC4wNDI1MDAwMDAwMDAwMDAwOSwiZHJpdmVyOm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYUltcHJvdmVtZW50VG9CYXNlOjEiOjAsImRyaXZlcjpwcm9qZWN0U2FsZXNHcm93dGgiOjAuMjIsImRyaXZlci1yYW5nZTpwcm9qZWN0U2FsZXNHcm93dGg6MCI6MC4xNSwiZHJpdmVyLXJhbmdlOnByb2plY3RTYWxlc0dyb3d0aDoxIjowLjMsImRyaXZlcjpvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDowIjowLjA2MDc2MDg2OTU2NTIxNzE5LCJkcml2ZXItcmFuZ2U6b3RoZXJTYWxlc0dyb3d0aDoxIjowLjA2NDM4NDA1Nzk3MTAxNDUzLCJkcml2ZXI6cHJvamVjdENvZ3NJbXByb3ZlbWVudEFmdGVyQmFzZSI6MC4wMTUsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjAiOjAsImRyaXZlci1yYW5nZTpwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlOjEiOjAuMDMsImRyaXZlcjpvdGhlckNvZ3NJbXByb3ZlbWVudCI6MC4wMDUsImRyaXZlci1yYW5nZTpvdGhlckNvZ3NJbXByb3ZlbWVudDowIjowLjAwNSwiZHJpdmVyLXJhbmdlOm90aGVyQ29nc0ltcHJvdmVtZW50OjEiOjAuMDA1MTM0NTc1NTY5MzU4MTk3NSwiZHJpdmVyOnByb2plY3RQYXlHcm93dGgiOjAuMDcsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjAiOjAuMDUsImRyaXZlci1yYW5nZTpwcm9qZWN0UGF5R3Jvd3RoOjEiOjAuMSwiZHJpdmVyOm90aGVyUGF5R3Jvd3RoIjowLjAyNDg0NjQ1ODQ2OTI0MDI3LCJkcml2ZXItcmFuZ2U6b3RoZXJQYXlHcm93dGg6MCI6MC4wMjQxMzk0NTcwMjM3MTc0NDQsImRyaXZlci1yYW5nZTpvdGhlclBheUdyb3d0aDoxIjowLjAyNTU1MzQ1OTkxNDc2MzA5NiwiZHJpdmVyOm90aGVyT2ZmaWNlclBheUdyb3d0aCI6MC4wNDUsImRyaXZlci1yYW5nZTpvdGhlck9mZmljZXJQYXlHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOm90aGVyT2ZmaWNlclBheUdyb3d0aDoxIjowLjA4LCJkcml2ZXI6cHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wNCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RIZWFkY291bnRHcm93dGg6MSI6MC4wOCwiZHJpdmVyOm90aGVySGVhZGNvdW50R3Jvd3RoIjowLjA0NTgzMzMzMzMzMzMzMzM4NiwiZHJpdmVyLXJhbmdlOm90aGVySGVhZGNvdW50R3Jvd3RoOjAiOjAuMDQ0MTY2NjY2NjY2NjY2NjgsImRyaXZlci1yYW5nZTpvdGhlckhlYWRjb3VudEdyb3d0aDoxIjowLjA0NzUwMDAwMDAwMDAwMDA5LCJkcml2ZXI6cHJvamVjdFNnYVJhdGVFbmQiOjAuMDE1LCJkcml2ZXItcmFuZ2U6cHJvamVjdFNnYVJhdGVFbmQ6MCI6MCwiZHJpdmVyLXJhbmdlOnByb2plY3RTZ2FSYXRlRW5kOjEiOjAuMDMsImRyaXZlcjpvdGhlclNnYVJhdGVFbmQiOjAuMDA1LCJkcml2ZXItcmFuZ2U6b3RoZXJTZ2FSYXRlRW5kOjAiOjAsImRyaXZlci1yYW5nZTpvdGhlclNnYVJhdGVFbmQ6MSI6MC4wMSwiZHJpdmVyOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1MzgwMTE2OTU5MDY0MzI1LCJkcml2ZXItcmFuZ2U6cHJvamVjdE9mZmljZXJQYXlHcm93dGg6MCI6MC4wNDI2MzE1Nzg5NDczNjgzNiwiZHJpdmVyLXJhbmdlOnByb2plY3RPZmZpY2VyUGF5R3Jvd3RoOjEiOjAuMDY1NTU1NTU1NTU1NTU1NTgsImRyaXZlcjppbnZlc3RtZW50IjoyMzAwMDAwLCJkcml2ZXItcmFuZ2U6aW52ZXN0bWVudDowIjoxNTAwMDAwLCJkcml2ZXItcmFuZ2U6aW52ZXN0bWVudDoxIjoyMDAwMDAwMCwiZHJpdmVyOnN1YnNpZHkiOjc2NjAwMCwiZHJpdmVyLXJhbmdlOnN1YnNpZHk6MCI6MTAwMDAwLCJkcml2ZXItcmFuZ2U6c3Vic2lkeToxIjo1MDAwMDAwLCJkcml2ZXI6bG9jYWxCZW5jaG1hcmsiOjIzLCJkcml2ZXItcmFuZ2U6bG9jYWxCZW5jaG1hcms6MCI6MCwiZHJpdmVyLXJhbmdlOmxvY2FsQmVuY2htYXJrOjEiOjEwMCwidGFyZ2V0OmNvbXBhbnlTYWxlc0NhZ3I6dmFsdWUiOjE1LCJ0YXJnZXQ6Y29tcGFueVNhbGVzQ2FncjptYXgiOjM1LCJ0YXJnZXQ6Y29tcGFueVNhbGVzSW5jcmVhc2U6dmFsdWUiOjgyNDAwMDAsInRhcmdldDpjb21wYW55UGF5U2NoZWR1bGU6dmFsdWUiOjMuNSwidGFyZ2V0OmNvbXBhbnlQYXlTY2hlZHVsZTptYXgiOjcsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTp2YWx1ZSI6NjAsInRhcmdldDpwcm9qZWN0U2FsZXNTaGFyZTptYXgiOjk1LCJ0YXJnZXQ6cHJvamVjdFNhbGVzQ2Fncjp2YWx1ZSI6MjIsInRhcmdldDpwcm9qZWN0U2FsZXNDYWdyOm1heCI6MzUsInRhcmdldDpwcm9qZWN0U2FsZXNJbmNyZWFzZTp2YWx1ZSI6NzQ4MDAwMCwidGFyZ2V0OmxhYm9yUHJvZHVjdGl2aXR5Q2Fncjp2YWx1ZSI6MjEsInRhcmdldDpsYWJvclByb2R1Y3Rpdml0eUNhZ3I6bWF4IjozNSwidGFyZ2V0OnZhbHVlQWRkZWRJbmNyZWFzZTp2YWx1ZSI6MTg3ODAwMCwidGFyZ2V0OmVtcGxveWVlUGF5Q2Fncjp2YWx1ZSI6NywidGFyZ2V0OmVtcGxveWVlUGF5Q2FncjptYXgiOjEwLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlJbmNyZWFzZTp2YWx1ZSI6Mjg1MDAwLCJ0YXJnZXQ6aW52ZXN0bWVudFNhbGVzUmF0aW86dmFsdWUiOjE1LCJ0YXJnZXQ6aW52ZXN0bWVudFNhbGVzUmF0aW86bWF4Ijo3MCwidGFyZ2V0OnZhbHVlQWRkZWRTdWJzaWR5UmF0aW86dmFsdWUiOjIxMywidGFyZ2V0OnZhbHVlQWRkZWRTdWJzaWR5UmF0aW86bWF4IjozNTAsInRhcmdldDpsb2NhbEJlbmNobWFyazp2YWx1ZSI6MjMsInRhcmdldDpsb2NhbEJlbmNobWFyazptYXgiOjQwLCJ0YXJnZXQ6b2ZmaWNlclBheUNhZ3I6dmFsdWUiOjYsInRhcmdldDpvZmZpY2VyUGF5Q2FncjptYXgiOjEwLCJ0YXJnZXQ6b2ZmaWNlclBheUluY3JlYXNlOnZhbHVlIjowLCJ0YXJnZXQ6Y29tcGFueVNhbGVzSW5jcmVhc2U6bWF4IjoyNTI2OTAwMCwidGFyZ2V0OnByb2plY3RTYWxlc0luY3JlYXNlOm1heCI6MTM2ODQwMDAsInRhcmdldDp2YWx1ZUFkZGVkSW5jcmVhc2U6bWF4IjozMzQzMDAwLCJ0YXJnZXQ6ZW1wbG95ZWVQYXlJbmNyZWFzZTptYXgiOjM3NDAwMH0sIm1ldHJpY0dyb3VwQmFzZXMiOnsiY29tcGFueVNhbGVzIjoicmF0ZSIsInByb2plY3RTYWxlcyI6InJhdGUiLCJsYWJvclByb2R1Y3Rpdml0eSI6InJhdGUiLCJlbXBsb3llZVBheSI6InJhdGUifSwiYXBwbGljYXRpb25DYXRlZ29yeSI6ImdlbmVyYWwiLCJhZGp1c3RlZERyaXZlcnMiOnsicHJvamVjdE1hcmtldEdyb3d0aCI6MC4wNSwicHJvamVjdENvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42Nzk5OTk5OTk5OTk5OTk5LCJvdGhlckNvZ3NSYXRlV2hlblNhbGVzWmVybyI6MC42Nzk5OTk5OTk5OTk5OTk5LCJwcm9qZWN0Q29nc1JhdGVUb0Jhc2UiOjAuNjgsIm90aGVyQ29nc1JhdGVUb0Jhc2UiOjAuNjgsInByb2plY3RFbXBsb3llZVNhbGFyeVNoYXJlIjowLjk1LCJvdGhlckVtcGxveWVlU2FsYXJ5U2hhcmUiOjAuOTUsInByb2plY3RPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwib3RoZXJPZmZpY2VyQ29tcGVuc2F0aW9uU2hhcmUiOjAuOSwicHJvamVjdENvZ3NEZXByZWNpYXRpb25TaGFyZSI6MC4yNSwib3RoZXJDb2dzRGVwcmVjaWF0aW9uU2hhcmUiOjAuMiwicHJvamVjdFJlc2VhcmNoRGV2ZWxvcG1lbnRSYXRlIjowLjAwNSwib3RoZXJSZXNlYXJjaERldmVsb3BtZW50UmF0ZSI6MC4wMDQsInByb2plY3ROb25PcGVyYXRpbmdSYXRlIjowLCJvdGhlck5vbk9wZXJhdGluZ1JhdGUiOi0wLjAwNSwicHJvamVjdEV4dHJhb3JkaW5hcnlSYXRlIjowLCJvdGhlckV4dHJhb3JkaW5hcnlSYXRlIjowLCJlZmZlY3RpdmVUYXhSYXRlIjowLjMsInByb2plY3RTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5NywicHJvamVjdEZpcnN0WWVhclNhbGVzIjowLCJwcm9qZWN0QmFzZVllYXJTYWxlcyI6MCwicHJvamVjdENvZ3NJbXByb3ZlbWVudFRvQmFzZSI6Ni41MjgxMTEzODQ3OTU5MjFlLTE3LCJwcm9qZWN0UGF5R3Jvd3RoVG9CYXNlIjowLjAyMDczNTk5NDE4MzE4OTE2NiwicHJvamVjdEhlYWRjb3VudEdyb3d0aFRvQmFzZSI6MC4wNTIyMDk2NTY4MTE3MDExMSwicHJvamVjdFNnYUltcHJvdmVtZW50VG9CYXNlIjowLCJwcm9qZWN0T2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNTQwOTM1NjcyNTE0NjE5Nywib3RoZXJTYWxlc0dyb3d0aFRvQmFzZSI6MC4wNDI1NzI0NjM3NjgxMTU4NTQsIm90aGVyQ29nc0ltcHJvdmVtZW50VG9CYXNlIjowLCJvdGhlclBheUdyb3d0aFRvQmFzZSI6MC4wMjA1NTM0NTk5MTQ3NjMwOTUsIm90aGVyT2ZmaWNlclBheUdyb3d0aFRvQmFzZSI6MC4wNCwib3RoZXJIZWFkY291bnRHcm93dGhUb0Jhc2UiOjAuMDQwNjI1MDAwMDAwMDAwMDUsIm90aGVyU2dhSW1wcm92ZW1lbnRUb0Jhc2UiOjAsInByb2plY3RTYWxlc0dyb3d0aCI6MC4yMjAyMDUyNzMxMjA2</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">c3Vic2lkeSI6NzY2MDAwLCJsb2NhbEJlbmNobWFyayI6MjN9fQ==</t>
+          <t xml:space="preserve">MDU3LCJvdGhlclNhbGVzR3Jvd3RoIjowLjA2MjU3MjQ2Mzc2ODExNTg2LCJwcm9qZWN0Q29nc0ltcHJvdmVtZW50QWZ0ZXJCYXNlIjowLjAxNSwib3RoZXJDb2dzSW1wcm92ZW1lbnQiOjAuMDA1LCJwcm9qZWN0UGF5R3Jvd3RoIjowLjA5MTU3MTE4NjI3MjU2NDk4LCJvdGhlclBheUdyb3d0aCI6MC4wMjQ4NDY0NTg0NjkyNDAyNywib3RoZXJPZmZpY2VyUGF5R3Jvd3RoIjowLjA0NSwicHJvamVjdEhlYWRjb3VudEdyb3d0aCI6MC4wMzczNDQ0NjQwMjgyMDA2MSwib3RoZXJIZWFkY291bnRHcm93dGgiOjAuMDQ1ODMzMzMzMzMzMzMzMzg2LCJwcm9qZWN0U2dhUmF0ZUVuZCI6MC4wMTUsIm90aGVyU2dhUmF0ZUVuZCI6MC4wMDUsInByb2plY3RPZmZpY2VyUGF5R3Jvd3RoIjowLjA1Mzc2NzAyODY1Mzg4MTUxLCJpbnZlc3RtZW50IjoyMzAwMDAwLCJzdWJzaWR5Ijo3NjYwMDAsImxvY2FsQmVuY2htYXJrIjoyM319</t>
         </is>
       </c>
     </row>

</xml_diff>